<commit_message>
fix(ai-insights): make ComprehensiveInsightsResponse.insights Optional (#42)
One-line schema fix closes Backlog #42. The error path in
get_comprehensive_insights (when _fetch_historical_prices returns None
or returns <20 rows) builds ComprehensiveInsightsResponse(insights=None)
but the schema previously declared insights as a non-Optional
ComprehensiveInsights, so the endpoint 500s on insufficient-data inputs
in production today.

Schema change:
  insights: ComprehensiveInsights
  -> insights: Optional[ComprehensiveInsights] = None

The two tests in test_comprehensive_insights.py that previously pinned
the broken behavior with pytest.raises(Exception) now assert the proper
response shape (status="error", insights=None).

ai-insights coverage holds at 91.9%; all 113 tests still pass; all 9
services still pass their CI floors.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -7833,12 +7833,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Surfaced during 2026-05-12 #66 coverage climb; insufficient data + missing-fetch paths both 500 today. Fix: mark insights Optional[ComprehensiveInsights] = None in ComprehensiveInsightsResponse schema</t>
+          <t>Surfaced during 2026-05-12 #66 coverage climb; insufficient data + missing-fetch paths both 500 today. Fix: mark insights Optional[ComprehensiveInsights] = None in ComprehensiveInsightsResponse schema | 2026-05-12: fixed via one-line schema change — insights field is now Optional[ComprehensiveInsights] = None. The 2 pinned pytest.raises tests now assert the proper error response shape (status="error", insights=None) instead of pinning the broken behavior.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -8427,7 +8427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9582,6 +9582,33 @@
       <c r="E43" t="inlineStr">
         <is>
           <t>Coverage tier 1 (&gt;=80%): chatbot 96%, ai-insights 92%, knowledge-qa 91%, analysis 91%, auth 87%, portfolio 84%, stock-data 83%, journal 80%. Tier 3 (&lt;60%): prediction 43%. 8 of 9 services across Phase 3 target — prediction is the last remaining. Open: #28 ESLint cleanup; #24 secret store; #42 ai-insights bug. Phase 5 P2 — backtesting UI, mobile, contract tests, i18n.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Backlog #42: ComprehensiveInsightsResponse — make insights Optional</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>#71 closes Backlog #42 with a one-line schema fix. ComprehensiveInsightsResponse now declares insights as Optional[ComprehensiveInsights] = None so the error path in get_comprehensive_insights (insufficient data, missing fetch) can return {status: 'error', insights: None} without tripping pydantic validation. Updated the 2 tests in test_comprehensive_insights.py that previously pinned the broken behavior with pytest.raises — they now assert the proper response shape: out.status == 'error', out.insights is None. All 113 ai-insights tests still pass; coverage holds at 91.9%. All 9 services still pass their CI floors.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Two tests originally written to pin the broken behavior in #66 now assert the corrected behavior. The 'pin the broken behavior with pytest.raises' pattern is a useful interim — it documents the bug, blocks silent fixes that don't update the test, and lets the fix PR show a clean before/after diff. Total Backlog #42 cost: 1 source line change + 2 test rewrites + ROADMAP entry. Total turnaround: &lt; 5 minutes from request to commit.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Open: prediction-service (43%) is the last service below 80% — would complete the 9-of-9 sweep. Then #28 ESLint cleanup, #24 secret store. Phase 5 P2 — backtesting UI, mobile, contract tests, i18n.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
frontend(lint): burn ESLint warnings to 0; flip CI to strict (#28)
Cleared all 114 lingering ESLint warnings across the React app
(unused imports/vars, array-callback-return, eqeqeq, template-string,
anonymous-default-export, exhaustive-deps) and switched frontend-ci
to strict mode: --max-warnings 0 on lint and CI=true on the CRA
production build. New warnings now fail the job.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -27,7 +27,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -126,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -152,6 +154,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7343,7 +7346,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -8427,7 +8430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9610,6 +9613,11 @@
         <is>
           <t>Open: prediction-service (43%) is the last service below 80% — would complete the 9-of-9 sweep. Then #28 ESLint cleanup, #24 secret store. Phase 5 P2 — backtesting UI, mobile, contract tests, i18n.</t>
         </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="n">
+        <v>46155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
frontend(prediction): add Backtest UI wrapping /predict/backtest
New /backtest page (Sidebar "Dự đoán" → Backtest) with a form for
symbol, model_type, date range, and prediction horizon. Submits to
POST /predict/backtest via modelService.runBacktest and renders the
returned accuracy stats: direction-accuracy bar, MAE/RMSE, average
confidence, and prediction counts.

The endpoint reports prediction accuracy, not strategy PnL — page
labelled "Prediction Backtest" to make the scope explicit. A PnL
strategy backtest can layer on top later.

Validated with 3 RTL tests (success / API error / invalid date
range); full suite 45/45 pass, lint clean, CI=true production
build compiles.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -5857,7 +5857,7 @@
       </c>
       <c r="F36" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G36" s="14" t="inlineStr"/>
@@ -8430,7 +8430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9617,6 +9617,11 @@
     </row>
     <row r="45">
       <c r="A45" s="15" t="n">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="n">
         <v>46155</v>
       </c>
     </row>

</xml_diff>

<commit_message>
frontend(journal): polish — carry-forward adjustments + today's plan card
Two cross-page wirings of existing journal data; no schema changes.

A. DailyPlanning shows a "Last Week's Adjustments" card pulled from
   the most recent WeeklyReview.key_adjustments for the selected
   account. Bullets split on newlines; card hides when empty.

B. TradeLog shows a "Today's Plan" card pulled from the DailyPlan
   whose plan_date matches today. Collapsible; shows new_trade_ideas
   and market_review. When today has no plan, renders a small CTA
   linking to DailyPlanning instead.

6 new RTL tests; full suite 51/51; lint clean; CI=true build OK.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -805,7 +805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4310,6 +4310,80 @@
       </c>
       <c r="F110" s="14" t="inlineStr"/>
       <c r="G110" s="14" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>WeeklyReview adjustments carried into DailyPlanning</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>src/components/Pages/Journal/DailyPlanning.js</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Fetches latest WeeklyReview; renders key_adjustments bullets above the editor. 3 RTL tests.</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Polish A; read-only carry-forward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Today's DailyPlan visible in TradeLog</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>src/components/Pages/Journal/TradeLog.js</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Renders today's new_trade_ideas + market_review (collapsible) or an empty CTA. 3 RTL tests.</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Polish B; no by-date endpoint; filters list client-side.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G110"/>
@@ -8430,7 +8504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9622,6 +9696,11 @@
     </row>
     <row r="46">
       <c r="A46" s="15" t="n">
+        <v>46155</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="n">
         <v>46155</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(roadmap): sync ROADMAP.xlsx + roadmap_version_2.xlsx after CD-6/7 completion
ROADMAP.xlsx:
- Feature Inventory: add chart-decomp Part I, Part II, PatternTab (all Done);
  fix stale statuses (alert evaluation, real LLM, training polling → Done;
  7 Migration items → Obsolete; useRouter Roadmap row → Done)
- Sessions Log #53: summarise CD-6 A6-A17 + CD-7 B1-B4 work
- Roadmap: add "Chart Decomposition & Pattern Detection" row → Done

roadmap_version_2.xlsx:
- Session Log: what's-next review + final CD sync entry
- All CD-1..CD-7 tasks confirmed Done; 3 open Feature Inventory items remain

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G113"/>
+  <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="E47" s="14" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F47" s="14" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="G47" s="14" t="inlineStr">
         <is>
-          <t>InsightsService is in-house heuristic today</t>
+          <t>Done — OPENAI/ANTHROPIC keys plumbed and used in InsightsService (Phase 4)</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3118,7 @@
       </c>
       <c r="E73" s="14" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="F73" s="14" t="inlineStr">
@@ -3126,7 +3126,11 @@
           <t>Listed in Phase 3 plan, not present</t>
         </is>
       </c>
-      <c r="G73" s="14" t="inlineStr"/>
+      <c r="G73" s="14" t="inlineStr">
+        <is>
+          <t>Obsolete 2026-05-06: Django fully retired.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="14" t="inlineStr">
@@ -3151,7 +3155,7 @@
       </c>
       <c r="E74" s="14" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="F74" s="14" t="inlineStr">
@@ -3161,7 +3165,7 @@
       </c>
       <c r="G74" s="14" t="inlineStr">
         <is>
-          <t>Audit completeness</t>
+          <t>Audit completeness | Obsolete 2026-05-06: Django fully retired.</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3192,7 @@
       </c>
       <c r="E75" s="14" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="F75" s="14" t="inlineStr">
@@ -3198,7 +3202,7 @@
       </c>
       <c r="G75" s="14" t="inlineStr">
         <is>
-          <t>Per-table sync coverage TBD</t>
+          <t>Per-table sync coverage TBD | Obsolete 2026-05-06: Django fully retired.</t>
         </is>
       </c>
     </row>
@@ -3225,7 +3229,7 @@
       </c>
       <c r="E76" s="14" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="F76" s="14" t="inlineStr">
@@ -3235,7 +3239,7 @@
       </c>
       <c r="G76" s="14" t="inlineStr">
         <is>
-          <t>Validate against current schemas</t>
+          <t>Validate against current schemas | Obsolete 2026-05-06: Django fully retired.</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3266,7 @@
       </c>
       <c r="E77" s="14" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="F77" s="14" t="inlineStr">
@@ -3270,7 +3274,11 @@
           <t>Phase 3.2</t>
         </is>
       </c>
-      <c r="G77" s="14" t="inlineStr"/>
+      <c r="G77" s="14" t="inlineStr">
+        <is>
+          <t>Obsolete 2026-05-06: Django fully retired.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="14" t="inlineStr">
@@ -3295,7 +3303,7 @@
       </c>
       <c r="E78" s="14" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="F78" s="14" t="inlineStr">
@@ -3305,7 +3313,7 @@
       </c>
       <c r="G78" s="14" t="inlineStr">
         <is>
-          <t>Validate end-to-end runbook</t>
+          <t>Validate end-to-end runbook | Obsolete 2026-05-06: Django fully retired.</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3340,7 @@
       </c>
       <c r="E79" s="14" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="F79" s="14" t="inlineStr">
@@ -3342,7 +3350,7 @@
       </c>
       <c r="G79" s="14" t="inlineStr">
         <is>
-          <t>Gate on 100% traffic + 2 weeks soak</t>
+          <t>Gate on 100% traffic + 2 weeks soak | Obsolete 2026-05-06: Django fully retired.</t>
         </is>
       </c>
     </row>
@@ -3840,7 +3848,7 @@
       </c>
       <c r="E95" s="14" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F95" s="14" t="inlineStr">
@@ -4421,6 +4429,102 @@
       <c r="G113" t="inlineStr">
         <is>
           <t>Committed: eb119d9a (Day1) + 646cea39 (Day2/3/F-006). 204 ai-insights tests green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>chart-decomp-service</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Part I: MODWT/EMD/VMD/CWT/HHT decomposition + Hurst + Coherence + HAR/VMD-HAR + backtest</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>stock_microservices/services/chart-decomp-service | chart_decomp lib (CD-1 to CD-5)</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Full library (chart-decomp-lib) + FastAPI service. 202 tests. CLI repaired (B1). Hurst stationary guard (B2). DM-stat wired (B3). Version provenance __version__ + get_versions() (B4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>chart-decomp-service</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Part II: Pattern Detection — H&amp;S, Double, Flag/Pennant, Triangle + null-FPR + pipeline facade</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>stock_microservices/services/chart-decomp-service | chart_decomp lib (CD-6 to CD-7)</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>A6-A17 complete: detectors, registry, null_fpr, run_pattern_pipeline, calibrate_denoise_swings. /patterns/* service endpoints. II.5.1-II.5.4 mandatory harnesses green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>ChartDecomp</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Pattern Detection tab (FR-VIZ-1/2): 3-panel view + detection report</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>src/components/Pages/ChartDecomp/index.js (PatternTab) | CD-617</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Panel1 raw/denoised, Panel2 swing skeleton H/L dots, Panel3 ReferenceArea per detection. FR-VIZ-2 report table: pattern/start/end/score/confirmed/null-pct95.</t>
         </is>
       </c>
     </row>
@@ -4467,7 +4571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -6384,7 +6488,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -6395,6 +6499,48 @@
       <c r="I46" t="inlineStr">
         <is>
           <t>Backlog #29</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Phase 4 — Polish &amp; gaps</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>chart-decomp</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Chart Decomposition &amp; Pattern Detection</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Part I: MODWT/EMD/VMD/CWT/HHT/Hurst/Coherence/HAR/VMD-HAR/backtest. Part II: H&amp;S, Double, Flag/Pennant, Triangle detectors + null-FPR + pipeline. Service /chart-decomp + /patterns endpoints. Frontend 5-tab page.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>you</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Full SRS delivered: CD-1..CD-5 (Part I), CD-6 A6-A17 (Part II), CD-7 B1-B4 (optional). 202 tests. CLI repaired. See roadmap_version_2.xlsx for per-task breakdown.</t>
         </is>
       </c>
     </row>
@@ -8543,7 +8689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9867,7 +10013,31 @@
           <t>orchestrator.py at 96%. Remaining 9 missing lines are the discipline-violations reason-chain append branch (only fires when violations list is non-empty — not exercised by the happy paths). Coverage tier 1 (&gt;=80%): chatbot 96%, ai-insights 92%, knowledge-qa 91%, analysis 91%, prediction 89%, decision-helper 91%, auth 87%, portfolio 84%, stock-data 83%, journal 80%. Open: #28 ESLint cleanup; #24 secret store. Phase 5 P2 — mobile responsive, contract tests, i18n.</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="15" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Chart Decomp CD-6 + CD-7: Part II pattern detection + optional tasks (roadmap_version_2.xlsx)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>A6-A17 + B1-B4 spanning 2026-05-30 to 2026-05-31. CD-6 (Part II): A6 H&amp;S+InvH&amp;S, A7 Double Top/Bottom, A8 Flag/Pennant, A9 Triangle asc/desc/sym, A10 default registry population, A11 null_fpr evaluator+is_noteworthy (FR-FPR-1/2), A12 run_pattern_pipeline facade+edge-flag (B6/C2), A13 calibrate_denoise_swings (FR-DN-2), A14 threshold-robustness harness (II.5.3, L4), A15 determinism harness (II.5.4/NFR-RP1), A16 /patterns/denoise|swings|detect|pipeline|null-fpr service endpoints, A17 PatternTab (FR-VIZ-1/2 three-panel + detection report table, en/vi i18n). CD-7 (optional): B1 CLI repair (stale calls + decompose/forecast/backtest/patterns subcmds), B2 Hurst stationary-input UserWarning, B3 dm_vs_har wired into metrics, B4 __version__ + get_versions() provenance. 202 Python tests pass. React build clean. roadmap_version_2.xlsx fully up to date.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>range_frac threshold is scale-robust across quiet/volatile regimes (II.5.3 proven). PyWavelets SWT requires N divisible by 2^level (N=500 → max level 2). Pattern detectors are purely geometric → deterministic (no RNG). null_fpr with fixed seed = II.5.4 compliance. Confirmed=False flag uses COI of finest kept MODWT band as edge_lag.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>All Chart Decomposition tasks complete. Next: Phase 3.5 hardening (p99 performance targets, HA/DR drill) | Prediction time-series CRUD verification | Secret store (#24) | Phase 5 mobile responsive + i18n</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
chore(roadmap): mark Phase 3.5 performance targets Done
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -5461,7 +5461,7 @@
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr"/>
@@ -5470,7 +5470,11 @@
           <t>you</t>
         </is>
       </c>
-      <c r="I21" s="14" t="inlineStr"/>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>Phase 3.5 SLA gate: thresholds.json (tiered p99: T2≤300ms, T1≤100ms, T3≤1000ms), test_basic_performance.py (p99 assertions), benchmark.py (standalone runner), performance-ci.yml (weekly + push CI gate). 2026-05-31.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
@@ -8689,7 +8693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10036,6 +10040,31 @@
       <c r="E53" t="inlineStr">
         <is>
           <t>All Chart Decomposition tasks complete. Next: Phase 3.5 hardening (p99 performance targets, HA/DR drill) | Prediction time-series CRUD verification | Secret store (#24) | Phase 5 mobile responsive + i18n</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="15" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Phase 3.5 performance SLA gate — p99 ≤ 300ms</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>thresholds.json updated to Phase 3.5 targets (T2 core p99≤300ms, T1 health p99≤100ms, T3 analysis p99≤1000ms). test_basic_performance.py rewritten: TestHealthSLA, TestCoreAPISLA, TestConcurrentSLA, TestThroughput, TestAnalysisSLA. benchmark.py: standalone runner, coloured terminal report, exit 0=all pass/1=violations/2=unreachable. performance-ci.yml: weekly + push trigger, starts docker-compose, runs benchmark, uploads JSON artifact.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Phase 3.5 SLA target is p99 ≤ 300ms for Tier-2 core APIs. T5 LLM endpoints (chatbot, ai-insights) are exempt — p99 ≤ 10s is appropriate there.</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Phase 3.5 performance targets Done. Next: HA + DR drill (P2) | Simulation dashboard (Partial) | Secret store (Partial) | Phase 5 mobile responsive.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(roadmap): mark Phase 3.5 HA + DR drill Done
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -5504,7 +5504,7 @@
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G22" s="14" t="inlineStr"/>
@@ -5513,7 +5513,11 @@
           <t>you</t>
         </is>
       </c>
-      <c r="I22" s="14" t="inlineStr"/>
+      <c r="I22" s="14" t="inlineStr">
+        <is>
+          <t>docker-compose.ha.yml (Swarm: replicas/anti-affinity/rolling/limits), production/kubernetes/deployment-ha.yaml (Deployments+PDB+HPA, maxUnavailable=0, podAntiAffinity, probes), scripts/backup.sh (MySQL+Redis RPO automation), scripts/dr-drill.sh (automated drill, measures RTO), production/docs/DR_RUNBOOK.md (RPO 1h/RTO 4h, recovery procedures). 25 validation tests. 2026-05-31.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
@@ -8693,7 +8697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10065,6 +10069,31 @@
       <c r="E54" t="inlineStr">
         <is>
           <t>Phase 3.5 performance targets Done. Next: HA + DR drill (P2) | Simulation dashboard (Partial) | Secret store (Partial) | Phase 5 mobile responsive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="15" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Phase 3.5 HA + DR drill</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>docker-compose.ha.yml: Swarm overlay (replicas auth=2/stock-data=3/portfolio=3/analysis=2/prediction=2/gateway=2, anti-affinity via max_replicas_per_node, zero-downtime start-first rolling + rollback, resource limits, restart_policy). production/kubernetes/deployment-ha.yaml: Deployments with maxUnavailable=0, podAntiAffinity, requests/limits, liveness+readiness+startup probes, PodDisruptionBudget + HPA per service. scripts/backup.sh: hourly MySQL dump + 5-min Redis RDB, retention, optional S3. scripts/dr-drill.sh: kills containers, measures RTO vs budget, verifies recovery + Redis durability + backup viability, volume-safe. production/docs/DR_RUNBOOK.md: RPO 1h/RTO 4h, replica topology, backup strategy, per-failure recovery, drill log, escalation. tests/ha/test_ha_dr.py: 25 static validation tests, all pass.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>docker compose (non-Swarm) rejects replicas+container_name; the HA overlay targets `docker stack deploy` where Swarm ignores container_name — documented in file header + runbook. K8s manifests are the production HA target; compose overlay is for Swarm/local multi-replica.</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Phase 3.5 fully Done (security audit + performance targets + HA/DR all complete). Next open: Phase 5 — mobile responsive (P2), i18n (P3), API contract tests (P2), ESLint cleanup (P2); or Frontend simulation dashboard (Partial); or secret store (#24 Partial).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(roadmap): mark simulation dashboard Done (/simulation/run shipped)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -3914,12 +3914,12 @@
       </c>
       <c r="E97" s="14" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F97" s="14" t="inlineStr">
         <is>
-          <t>Empty state shown when no results</t>
+          <t>POST /simulation/run implemented (SimulationService); frontend was already complete. 18 backend tests.</t>
         </is>
       </c>
       <c r="G97" s="14" t="inlineStr">
@@ -8697,7 +8697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10094,6 +10094,31 @@
       <c r="E55" t="inlineStr">
         <is>
           <t>Phase 3.5 fully Done (security audit + performance targets + HA/DR all complete). Next open: Phase 5 — mobile responsive (P2), i18n (P3), API contract tests (P2), ESLint cleanup (P2); or Frontend simulation dashboard (Partial); or secret store (#24 Partial).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="15" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Simulation dashboard — implement backend /simulation/run</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Root cause: SimulationDashboard.js was fully built but prediction-service exposed only /simulation/{models,trained-solutions} — the Run button 404d on the missing /simulation/run. Added SimulationService.run_simulation: fetch OHLCV [start-400d,end], reuse PredictionService feature prep, train chosen model family on pre-start rows (causal), walk-forward predict next-day close, threshold trading engine (buy/sell/position_size), portfolio metrics (return, win rate, Sharpe, max drawdown, alpha vs buy&amp;hold) + prediction accuracy (direction, MAPE). SimulationRequest/Result schemas match the frontend shape. POST /simulation/run route (422 on SimulationError). 18 new tests, all pass; 61 related route tests still green.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Frontend payload already matched (thresholds sent as pct/100 = fractions). Pretrained-model path falls back to training a fresh model of the requested family (loading arbitrary saved estimators is environment-dependent / out of scope).</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Simulation dashboard now end-to-end functional. Remaining open: Phase 5 — mobile responsive (P2), i18n (P3), API contract tests (P2), ESLint cleanup (P2); secret store (#24 Partial); portfolio recommendations (Planned).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(roadmap): mobile-responsive foundation done; pass now In Progress
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -6000,7 +6000,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G34" s="14" t="inlineStr"/>
@@ -6009,7 +6009,11 @@
           <t>you</t>
         </is>
       </c>
-      <c r="I34" s="14" t="inlineStr"/>
+      <c r="I34" s="14" t="inlineStr">
+        <is>
+          <t>Foundation landed 2026-05-31: src/styles/responsive.css (overflow guards, fluid media, responsive-grid utilities, table-scroll, touch targets, header fixes) + layout.css header-title regression fix. Layout shell already responsive. Remaining: per-page audit to migrate 12 inline-gridTemplateColumns pages onto the new utilities.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
@@ -8697,7 +8701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10119,6 +10123,31 @@
       <c r="E56" t="inlineStr">
         <is>
           <t>Simulation dashboard now end-to-end functional. Remaining open: Phase 5 — mobile responsive (P2), i18n (P3), API contract tests (P2), ESLint cleanup (P2); secret store (#24 Partial); portfolio recommendations (Planned).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Phase 5 mobile-responsive — foundation pass</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Added src/styles/responsive.css (imported last in App.js): global overflow-x guards, fluid media, .responsive-grid-2/3/4/auto utilities (collapse at 1023/768px), .table-scroll wrapper, mobile page padding, touch targets (≥40px controls, 16px inputs to stop iOS zoom), header fixes + small-screen search collapse. Fixed layout.css header-title regression (28px→18px on mobile). Build clean; rules verified in CSS bundle.</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Layout shell was already responsive (fixed-drawer sidebar, hamburger, overlay, 1024px breakpoint). Inline gridTemplateColumns (12 files) cannot be overridden by CSS media queries — those need per-page migration to the utility classes. Backend down + no Playwright, so live screenshot verification deferred to when the stack is up.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Foundation done; mobile responsive now In Progress. Next: per-page audit (migrate inline-grid pages to .responsive-grid-*, wrap wide tables in .table-scroll), then visual check at 375/768px.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(roadmap): frontend rebuilt+redeployed, responsive foundation verified live
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8701,7 +8701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10148,6 +10148,31 @@
       <c r="E57" t="inlineStr">
         <is>
           <t>Foundation done; mobile responsive now In Progress. Next: per-page audit (migrate inline-grid pages to .responsive-grid-*, wrap wide tables in .table-scroll), then visual check at 375/768px.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Mobile-responsive foundation — rebuilt + redeployed frontend, verified live</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Rebuilt stockpredict-frontend image (docker compose -p stockpredict -f docker-compose.full-stack.yml build frontend) and recreated stock_frontend container. Confirmed responsive.css rules present in the LIVE served bundle (header-title:18px, responsive-grid-auto, table-scroll). Verified no horizontal overflow at a true 390px viewport via same-origin iframe DOM probe (scrollWidth==clientWidth==390) and a forced-390px-iframe screenshot (login card fits with even margins, all controls visible). Desktop (1280px) renders correctly. Diagnosed earlier "cut-off" screenshots as a headless-chrome minimum-window-width clamping artifact, not a real overflow.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>google-chrome --headless --window-size=390 clamps to a ~500px minimum and crops the screenshot, which falsely looks like overflow. Authoritative check is a forced-width iframe + documentElement.scrollWidth (same-origin) or a forced-width-iframe screenshot.</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Responsive foundation now LIVE on stock_frontend (port 3004) and verified. Remaining: per-page audit — migrate the 12 inline-gridTemplateColumns pages to .responsive-grid-* and wrap wide tables in .table-scroll, verified on authenticated pages.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(roadmap): mobile-responsive pass complete — audit live + verified
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -6000,7 +6000,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G34" s="14" t="inlineStr"/>
@@ -6011,7 +6011,7 @@
       </c>
       <c r="I34" s="14" t="inlineStr">
         <is>
-          <t>Foundation landed 2026-05-31: src/styles/responsive.css (overflow guards, fluid media, responsive-grid utilities, table-scroll, touch targets, header fixes) + layout.css header-title regression fix. Layout shell already responsive. Remaining: per-page audit to migrate 12 inline-gridTemplateColumns pages onto the new utilities.</t>
+          <t>Done 2026-05-31. Foundation (responsive.css: overflow guards, fluid media, grid utilities, table-scroll, touch targets, header fixes) + per-page audit (12 inline grids → .responsive-stack/.responsive-stack-2up overrides; global mobile table rule for ~29 table pages; CSS-file grids already responsive). Rebuilt+redeployed stock_frontend and verified live: override rules in served bundle + 390px screenshot shows inline 2/4-col grids stacking, 800px preserves desktop layout.</t>
         </is>
       </c>
     </row>
@@ -8701,7 +8701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10173,6 +10173,31 @@
       <c r="E58" t="inlineStr">
         <is>
           <t>Responsive foundation now LIVE on stock_frontend (port 3004) and verified. Remaining: per-page audit — migrate the 12 inline-gridTemplateColumns pages to .responsive-grid-* and wrap wide tables in .table-scroll, verified on authenticated pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Mobile-responsive per-page audit — done + verified live</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Migrated 12 fixed-column inline grids to .responsive-stack/.responsive-stack-2up (author !important overrides non-important inline styles on mobile; desktop untouched): PositionCalculator, Backtest, RiskDashboard, AnalyticsPage, DisciplineDashboard, DecisionConsole, RiskPrefsPanel, TradePlanModal. Added global .page-content table mobile rule (display:block+overflow-x:auto) covering ~29 table pages. auto-fill grids + CSS-file grids already responsive (verified). Rebuilt + redeployed stock_frontend; confirmed exact override rules in live CSS bundle; live-CSS test page screenshot proves inline 2-col and 4-col grids stack at 390px and preserve layout at 800px.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Author !important beats non-important inline styles — the key to reflowing inline grids without restructuring JSX (just add a className, keep the inline style for desktop).</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Phase 5 mobile-responsive pass COMPLETE (foundation + audit, live + verified). Remaining Phase 5: i18n (P3), API contract tests (P2), ESLint cleanup (P2).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(roadmap): ESLint cleanup done — strict frontend gate green
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -6458,7 +6458,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -6468,7 +6468,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Gates strict CI; informational today</t>
+          <t>Done 2026-05-31: cleared the final 11 warnings (6 no-unused-vars, 4 exhaustive-deps, 1 anonymous-default-export). CI=true npm run build now compiles clean; frontend-ci strict gate green.</t>
         </is>
       </c>
     </row>
@@ -7622,7 +7622,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>frontend-ci stays informational until clean; gates strict mode | 2026-05-07: 9 anonymous-default-export warnings fixed (services/*); CI workflow now uses CI=false on build step so warnings dont break the gate. Remaining ~98 warnings (mostly unused imports) are incremental cleanup.</t>
+          <t>frontend-ci stays informational until clean; gates strict mode | 2026-05-07: 9 anonymous-default-export warnings fixed (services/*); CI workflow now uses CI=false on build step so warnings dont break the gate. Remaining ~98 warnings (mostly unused imports) are incremental cleanup. | 2026-05-31: final 11 warnings cleared; CI=true build compiles clean — strict gate fully green.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -8701,7 +8701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10198,6 +10198,31 @@
       <c r="E59" t="inlineStr">
         <is>
           <t>Phase 5 mobile-responsive pass COMPLETE (foundation + audit, live + verified). Remaining Phase 5: i18n (P3), API contract tests (P2), ESLint cleanup (P2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="15" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ESLint cleanup — strict CI gate green</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Cleared all 11 remaining frontend ESLint warnings: 6 no-unused-vars (fmt1, two `const N`, useCallback import, TrendingDown import, loadingWl binding), 4 react-hooks/exhaustive-deps (run-once effects → eslint-disable-next-line with intent), 1 import/no-anonymous-default-export (chartDecompService). CI=true npm run build now compiles clean. frontend-ci.yml already uses CI=true, so the strict gate is green again (these warnings had been breaking it).</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>frontend-ci was already strict (CI=true); the backlog note about CI=false was stale. Fixing the 11 warnings was what actually unblocked the strict gate.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ESLint cleanup done. Remaining Phase 5: Vietnamese i18n (P3), API contract tests (P2).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(roadmap): i18n vi gaps closed + verified live
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -6125,7 +6125,7 @@
       </c>
       <c r="F37" s="14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G37" s="14" t="inlineStr"/>
@@ -6136,7 +6136,7 @@
       </c>
       <c r="I37" s="14" t="inlineStr">
         <is>
-          <t>Suggestions and intents already in vi</t>
+          <t>Done 2026-05-31. react-i18next already wired with full en/vi parity (2102 keys) + working EN|VI switcher. Closed content gaps: translated 30 English-identical UI labels + page titles to Vietnamese (acronyms/jargon/product names correctly left). Rebuilt+redeployed stock_frontend; verified all new VI strings present in live JS bundle.</t>
         </is>
       </c>
     </row>
@@ -8701,7 +8701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10223,6 +10223,31 @@
       <c r="E60" t="inlineStr">
         <is>
           <t>ESLint cleanup done. Remaining Phase 5: Vietnamese i18n (P3), API contract tests (P2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="15" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>i18n — closed vi content gaps, verified live</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>react-i18next was already mature: full en/vi leaf-key parity (2102 each), working LanguageDetector + EN|VI switcher. Found 116 strings where vi == en; translated the 30 genuinely-translatable ones (19 metric/UI labels + 11 page titles, emphasis kept as valid trailing substring), left acronyms/jargon/product-names/placeholders/Long-Short. Identical 116→80. Rebuilt + redeployed stock_frontend; verified all 11 sampled VI strings in the live JS bundle (minifier unicode-escapes them, so check via escaped form). Build also shipped the ESLint cleanup.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>CRA imports locale JSON inline and the minifier unicode-escapes non-ASCII — verify bundled non-Latin strings by their \uXXXX escaped form, not the literal UTF-8.</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>i18n done + live. Phase 5 remaining: API contract tests (Pact/schemathesis, P2). Lower-priority leftovers: portfolio recommendations (Planned), secret store (#24 Partial).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(frontend): light-theme the AI Assistant submenus
Knowledge QA and Chatbot Agent shipped with their own off-theme
palettes (KQA hardcoded dark; Chatbot a purple gradient). Rewrite both
stylesheets onto the canonical light tokens from src/index.css :root.

- knowledge-qa.css: dark #0f1117/#161822/#1e2030 -> var(--paper)/
  --panel/--sidebar; teal #14b8a6 accent -> var(--pos); assistant
  bubbles get a var(--line) border; error banner -> light tint.
- chatbot-agent.css: drop the #667eea->#764ba2 gradient; panels on
  var(--paper)+var(--line); accent -> var(--pos); meta chip uses the
  dashboard buy-tint; container height -> calc(100vh - 64px).

CSS-only; components already use these class names. Update ROADMAP
Sessions Log.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8923,7 +8923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10553,6 +10553,34 @@
         </is>
       </c>
       <c r="F64" s="4" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>AI Assistant submenus light-theme pass (Knowledge QA + Chatbot Agent)</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Rewrote two standalone dark/branded stylesheets onto the app light theme (tokens from src/index.css :root). (1) src/styles/knowledge-qa.css: dark palette #0f1117/#161822/#1e2030 -&gt; var(--paper)/--panel/--sidebar; borders -&gt; var(--line); text -&gt; var(--ink)/--ink2/--ink3; teal #14b8a6 -&gt; var(--pos) (#2C5F4A) on user bubble/send btn/focus ring/score chip/icons/cursor; assistant bubbles gained var(--line) border; error banner -&gt; light tint #FBEAEA/var(--neg). (2) src/styles/chatbot-agent.css: replaced the #667eea-&gt;#764ba2 purple gradient throughout — container/header/pills/panels -&gt; var(--panel)+var(--line) on var(--paper); user bubble + active pill + send btn + suggestion hover + typing dots + strong text -&gt; var(--pos); bot bubble -&gt; var(--paper)+border; meta chip -&gt; dashboard buy-tint #E8EFE9; error -&gt; #FBEAEA/var(--neg); container height 100vh -&gt; calc(100vh - 64px) to fit under the app header. Both CSS-only; no JS changes (components already use these class names).</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Two AI-Assistant submenus shipped with their own off-theme palettes (KQA dark, Chatbot purple-gradient). Standardised both on the canonical light tokens and reused var(--pos) as the single accent green (already the app-wide active/link colour) plus the dashboard #E8EFE9 buy-tint, so the AI section now reads consistently with dashboard/auth/layout.</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>Done; CSS-only. Next: visually confirm both screens in browser, then commit. AI-Assistant submenu theme audit complete (KnowledgeQAChat + ChatbotAgent were the two off-theme screens).</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
fix(frontend): theme-ui must not flatten market-semantic cell colors
The centralized theme set `color` on every `.page-content td` /
`.rdt_TableCell`, which overrode class-based up/down/ceiling/floor/
reference colors on stock tables — those colors carry market meaning and
must be preserved.

- Drop `color` from the generic cell rules; cell text color is left to
  inherit / to component classes & inline styles. Keep only structural
  theming (padding/border-bottom/font-size).
- Add a hard exclusion that re-asserts the PriceBoard's own dark surface
  (.services .custom-table) so no theme rule can ever bleed into the
  trading-terminal grid, regardless of future specificity changes.

Rebuilt the frontend container and verified the served bundle sets no
color on generic cells and includes the priceboard guard.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8923,7 +8923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10609,6 +10609,34 @@
         </is>
       </c>
       <c r="F66" s="4" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Fix: theme-ui must not flatten market-semantic cell colors</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>theme-ui.css regression fix. Removed color from the generic .page-content td and .rdt_TableCell rules — cell text color must inherit / come from component classes &amp; inline styles, since stock screens encode market meaning (ceiling/floor/reference, up/down) in cell color. Added a HARD EXCLUSION block re-asserting the PriceBoard surface (.page-content .services .custom-table th/td -&gt; #0F0F0F cells, #1a365d gradient header, transparent rows) so no theme rule can bleed into the dark trading-terminal grid even if specificity changes later. Generic cells keep only structural theming (padding/border-bottom/font-size).</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>PriceBoard cell colors are inline &lt;span style&gt; on a dark .services bg (already specificity-protected), but the broader bug was .page-content td{color} flattening class-based up/down colors on other stock tables. Principle: never set cell text color in a global theme for a trading app. Rebuilt frontend container (docker compose up -d --build frontend); verified served bundle has no color on generic cells and the priceboard guard is present; container healthy on :3004.</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Done, rebuilt &amp; verified live on :3004. Commit + merge to main pending. No further theme work queued.</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(roadmap): log B7 live-verification + redeploy session
Record the deploy of chart-decomp-service + frontend from committed B7 code and
the end-to-end verification of /patterns/multiscale through the gateway. Note
deploy-interactive.sh needs no B7 change.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10786,6 +10786,34 @@
         </is>
       </c>
       <c r="F71" s="4" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Chart-decomp B7: live-verify /patterns/multiscale + redeploy</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Rebuilt + restarted stock_chart_decomp_service and stock_frontend from the committed B7 code via docker compose -f docker-compose.full-stack.yml build/up -d (both were week-old images). Verified /patterns/multiscale end-to-end through the Traefik gateway (host :18004, prefix /stock_helper/api/v2/chart-decomp): compute_fpr=False returns denoised_by_scale (3 scales) + roots + forest-preorder detections with scale/bias/parent_label; compute_fpr=True returns per-scale fpr_by_pattern_by_scale + spurious_nesting_fpr + noteworthy/null_percentile. Confirmed frontend bundle (main.8acdd466.js, :3004) contains B7 markers (patternMultiScale, patterns/multiscale, ms_toggle, panel_nested_title).</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>deploy-interactive.sh (in parent /home/tuanph/TuanPH/all_projects/) needs NO change for B7 — it already runs docker compose -f docker-compose.full-stack.yml -p stockpredict up -d --build, rebuilding chart-decomp-service + frontend; B7 added no new service/port/env/compose change. Running containers were stale (7-day / 2-day images) so a rebuild was required to pick up new code — a general gotcha after any code change.</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Part B fully shipped &amp; verified live (endpoint + UI). Remaining: human browser click-through of the PatternTab multi-scale view (cannot be automated here).</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(guide): bilingual user guide for Chart Decomposition + Decision Tools
Add docs/USER_GUIDE_chart_decomp_and_decision_tools.md — a VI/EN end-user
guide. Part 1 covers Analysis > Chart Decomposition (all 5 tabs). Part 2
covers all 12 Decision Tools sub-menus. Each section gives Benefit/Goal +
How-to steps, with TOC, glossary, and recommended daily workflow. UI labels
sourced from Sidebar.js and i18n locales so names match the live UI.

Log session row in ROADMAP.xlsx Sessions Log.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10814,6 +10814,33 @@
         </is>
       </c>
       <c r="F72" s="4" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>User docs: Chart Decomposition + Decision Tools guide (bilingual)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Added docs/USER_GUIDE_chart_decomp_and_decision_tools.md — a bilingual (VI/EN) end-user guide. Part 1 covers the Analysis &gt; Chart Decomposition page (all 5 tabs: Signal Decomposition, Time-Frequency, Hurst &amp; Coherence, Volatility Forecast, Pattern Detection incl. multi-scale). Part 2 covers all 12 Decision Tools sub-menus (Overview, Decision Console, Watchlist Board, Backtest Studio, Discipline, Scheduled Runs, Scanner, Heat Map, Analytics, Open Positions, Trade Outcomes, Risk Dashboard). Each section gives Benefit/Goal + How-to steps, with a TOC, glossary, and recommended daily workflow.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Pulled exact UI labels (EN+VI) from Sidebar.js and i18n locales en.json/vi.json so menu names match what users see. Doc is end-user oriented (benefits + click-steps), not API/code detail. Example numbers flagged as illustrative.</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Guide is complete and committed. Next: optionally extend with screenshots, or add guides for remaining menus (Portfolio, Journal, AI Insights).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(guide): bilingual user guide for Portfolio, Journal + AI Insights
Add docs/USER_GUIDE_portfolio_journal_ai_insights.md — a VI/EN end-user
guide. Part 1 covers the Portfolio menu (Holdings, Performance, Price
Alerts, Watchlist). Part 2 covers the Trade Journal menu's 6 sub-menus
(Dashboard, Accounts, Trade Log, Trade Diary, Daily Planning, Weekly
Review) around the Schwager method. Part 3 covers AI Insights (setup, the
5 result sections, technical-indicators chart). Each section gives
Benefit/Goal + How-to steps with a TOC. UI labels sourced from Sidebar.js
and i18n locales. Companion to the chart-decomp/decision-tools guide.

Log session row in ROADMAP.xlsx Sessions Log.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10839,6 +10839,33 @@
       <c r="E73" t="inlineStr">
         <is>
           <t>Guide is complete and committed. Next: optionally extend with screenshots, or add guides for remaining menus (Portfolio, Journal, AI Insights).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>User docs: Portfolio + Journal + AI Insights guide (bilingual)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Added docs/USER_GUIDE_portfolio_journal_ai_insights.md — bilingual (VI/EN) end-user guide. Part 1 Portfolio (Holdings, Performance, Price Alerts, Watchlist); Part 2 Trade Journal (Dashboard, Accounts, Trade Log, Trade Diary, Daily Planning, Weekly Review) framed around the Schwager method; Part 3 AI Insights (setup, the 5 result sections: confidence/sentiment/risk/patterns/predictions, and the technical-indicators chart). Each section gives Benefit/Goal + How-to steps, with TOC.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Same format and bilingual style as the prior chart-decomp/decision-tools guide. UI labels pulled from Sidebar.js + i18n en.json/vi.json so names match the live UI. Companion to docs/USER_GUIDE_chart_decomp_and_decision_tools.md.</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Guide complete and committed. Remaining menus without a user guide: Stocks, Market Movers, Prediction, Simulation, Chatbot/Knowledge-QA, Technical/Fundamental analysis, Decision Tools (already covered) — extend on request.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(health): readiness probe false 503 under SQLAlchemy 2.0
The /health/ready probe in 6 services ran `await conn.execute("SELECT 1")`
with a raw string. SQLAlchemy 2.0 rejects that with ObjectNotExecutableError,
and the except block misreported it as `database: disconnected` -> HTTP 503,
even though the DB was connected. Docker healthchecks use /health/live (process
liveness) so containers still showed "healthy", masking the broken probe.

Wrap the statement in `text("SELECT 1")` and add `from sqlalchemy import text`
where missing. Services: stock-data, analysis, auth, prediction, journal,
portfolio. decision-helper already used text() correctly.

After rebuild, all 6 return /health/ready 200. (knowledge-qa's 503 is a
separate, genuine issue: host Neo4j at host.docker.internal:7687 is not
running -- an optional Graph RAG dependency, left as-is.)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10893,6 +10893,33 @@
       <c r="E75" t="inlineStr">
         <is>
           <t>BID training should now run from the default 2y window. Existing BID solution still has NULL dates in DB but is handled gracefully client-side. Optional follow-up: persist sensible default training dates at solution-create time (SolutionAddNew).</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Bugfix: /health/ready false 503 (SQLAlchemy 2.0 raw-string execute)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Readiness probes in 6 services ran await conn.execute("SELECT 1") with a raw string, which SQLAlchemy 2.0 rejects with ObjectNotExecutableError; the except block misreported it as database disconnected, so /health/ready returned 503 even though the DB was connected (docker /health/live still passed, so containers showed healthy). Fixed by wrapping in text() and adding from sqlalchemy import text where missing. Services: stock-data, analysis, auth, prediction, journal, portfolio (prediction already imported text). decision-helper already used text() correctly; knowledge-qa 503 is a separate, genuine issue (host Neo4j at host.docker.internal:7687 not running - optional Graph RAG dependency).</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>docker healthcheck uses /health/live (process up) while /health/ready checks the DB - so a broken readiness probe hides behind a green docker status. Verified pre-fix in-container: raw string FAILs ObjectNotExecutableError, text("SELECT 1") returns 1. Rebuilding the 6 services to pick up the fix.</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>After rebuild, re-probe all /health/ready expecting 200 on the 6. knowledge-qa needs host Neo4j+Ollama (--profile gpu/cpu) to go ready - left as-is.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(solutions): unify Training/Prediction charts into one panel
The Solution Training and Prediction tabs rendered react-financial-charts
with several stacked sub-panels (price + each oscillator + volume). Replace
both FinancialTrainingChart and FinancialPredictionChart with one shared
UnifiedFinancialChart, consistent with the Company chart (StockChart):

- Single chart content (one pane), not 3 stacked sub-charts.
- Price-scale series (close/actual/predicted/validation/MA family/Bollinger)
  on the LEFT y-axis; indicators (RSI/MACD/CCI/Stochastic/ADX/ATR) overlaid
  on the RIGHT y-axis.
- Volume drawn inverted below the date axis via Chart flipYScale.
- "Series" checkbox dropdown (grouped Price / Indicators / Volume) toggles
  each line; oscillators default off since they share one right axis.

Remove the now-unused StraightLine import. eslint + CRA production build
both pass; frontend rebuilt and redeployed.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10920,6 +10920,33 @@
       <c r="E76" t="inlineStr">
         <is>
           <t>After rebuild, re-probe all /health/ready expecting 200 on the 6. knowledge-qa needs host Neo4j+Ollama (--profile gpu/cpu) to go ready - left as-is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Chart UX: unify Solution Training/Prediction charts to single panel</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Replaced the two multi-panel react-financial-charts components (FinancialTrainingChart / FinancialPredictionChart) in SolutionModal.js with one shared UnifiedFinancialChart: a single chart content where price-scale series (close/actual/predicted/validation/SMA/EMA/DEMA/TEMA/WMA/PSAR/Bollinger) sit on the LEFT y-axis, indicators (RSI/MACD/CCI/Stoch/ADX/ATR) overlay on the RIGHT y-axis, and volume is drawn inverted below the date axis (flipYScale). Added a Series checkbox dropdown (grouped Price/Indicators/Volume) to toggle each line; oscillators default off (shared right axis). Removed now-unused StraightLine import. Both tabs render the same component for consistency with the Company chart (StockChart.js) style requested by the user.</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>react-financial-charts Chart supports flipYScale (used for inverted volume) and overlaid panes with axisAt=right share the same origin/height as the price pane. CRA build treats warnings as errors (CI), so removed the orphaned StraightLine import; eslint + npm run build both pass. Frontend rebuilt+redeployed (bundle main.72424c4f.js).</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Charts unified + deployed. Pending user visual confirmation of inverted-volume placement and right-axis readability; tweak if needed. Same pattern could later be applied to other multi-panel charts for full app consistency.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(solutions): full target line in training chart, drop duplicate close series
The train endpoint computed predictions for every row (all_pred =
ml_model.predict(X)) but only stored predicted_price for the validation
tail, so the training portion (~80% of the chart) had no target line and
the user effectively saw only the source price. Fill predicted_price for
the whole window and expose validation_price separately for the
out-of-sample tail.

In the training-data mapping, `close` equals `actual`, so emitting both
drew two identical overlapping lines and a redundant Close toggle. Omit
`close`; the chart falls back to `actual` for volume coloring and the
edge indicator.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11001,6 +11001,33 @@
       <c r="E79" t="inlineStr">
         <is>
           <t>AI Insights chart fixed + deployed. Pending user visual confirmation. Follow-up: ai-insights mock fallback still emits CamelCase (handled via fallbacks); could normalize it. Consider migrating any other bespoke chart to the shared component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Fix Solution Training chart: missing target series + non-working toggles</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Root cause was backend, not the chart. prediction-service solution_routes.py _run_training computes all_pred=ml_model.predict(X) for every row but the chart payload stored predicted_price only for the validation tail (float(all_pred[i]) if is_validation else None), so ~80% (training portion) had no target line and the user saw essentially only the source price. The 'checkboxes do nothing' report was a side effect: the only price-scale series present were close and actual, which are identical values drawn on top of each other, so toggling one looked like nothing changed. Fix (solution_routes.py ~line 472): predicted_price now filled for the whole window (continuous fitted/target line) and added validation_price = all_pred for the out-of-sample tail only, so the validation segment can be toggled/highlighted distinctly. Frontend already maps both (processTrainingResults: predicted&lt;-predicted_price, validation&lt;-validation_price) and the shared UnifiedFinancialChart already does the requested layout (left axis = source/target/SMA/EMA/PSAR/Bollinger, right axis = RSI/MACD/Stoch/MFI/ATR, inverted volume bars), so no frontend change needed. Verified train API otherwise returns enough data: actual_price/close, indicators keyed by d.isoformat() (rsi, macd/signal/histogram, psar, bb_*, sma, ema...), volume. Rebuilt+restarted prediction-service (healthy); frontend image already current (build cache hit).</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>The train endpoint already merged indicators and source correctly; the only data gap was the target line restricted to the validation tail. Kept MACD on the right/oscillator axis (per user confirm) — MACD magnitude is tiny vs VND price so it would flat-line on the price axis. UnifiedFinancialChart only lists series actually present in data, so identical overlapping close/actual lines made toggles look broken; a distinct target line resolves that perception. Reopen path is fine: SolutionList fetches GET /solutions/{id} which json.loads training_result into an object.</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Backend fix deployed (prediction-service healthy). Pending user visual confirmation that target line + working toggles now appear after retraining a solution. Note latent issue: GET /solutions/all omits training_result, but modal opens via getSolutionById so restore works. Optional cleanup: training data emits both close and actual identically (redundant overlapping lines).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(chart-decomp): add bilingual Overview tab explaining the pipeline
Adds a new default "Overview" tab to the Chart Decomposition page so users
understand the goal and benefit before using the analytical tabs. Renders a
hero intro, goal card, benefits checklist, and a 5-stage pipeline (Signal
Decomposition -> Time-Frequency -> Hurst & Coherence -> Volatility Forecast ->
Pattern Detection) where each stage reveals a description + benefit on hover and
jumps to its tab on click. Hides the ticker input panel on the Overview tab.

Fully i18n via existing react-i18next infra (EN/VI) — new chart_decomp.overview.*
keys in both locale files; no new language toggle needed. Includes an RTL smoke
test covering EN/VI render, hover reveal, and input-panel visibility.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11082,6 +11082,33 @@
       <c r="E82" t="inlineStr">
         <is>
           <t>Prediction chart consistency deployed. Pending user confirmation that the Predict tab now shows indicators + volume + history context + forecast line like Training. Note: future points carry no indicators/volume (only the forecast close), by design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Make Chart Decomposition screen self-explanatory (Overview tab)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Added a new first tab "Overview" to the Chart Decomposition page (stock_react_javascript/.../components/Pages/ChartDecomp/index.js). New OverviewTab component renders a static "what is this &amp; why" page: hero intro, goal card, benefits checklist, and a horizontal 5-stage pipeline (Signal Decomposition -&gt; Time-Frequency -&gt; Hurst &amp; Coherence -&gt; Volatility Forecast -&gt; Pattern Detection) with ArrowRight connectors. Each stage card has an onMouseEnter/Leave hover reveal that expands to show a brief description + green benefit callout, plus a methods footer; clicking a stage jumps to that tab (onJump=setActiveTab). Default activeTab changed decomp-&gt;overview. Added lucide icons Info/ArrowRight/Check. Fully i18n: new chart_decomp.overview.* block (hero, goal, pipeline, per-stage stages.{key}.{title,role,desc,benefit,methods}, benefits[] array via returnObjects, cta) plus tabs.overview label added to BOTH en.json and vi.json. Language switching works through the existing react-i18next LanguageSwitcher (EN|VI) - no new mechanism needed.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>The app already has full react-i18next vi/en infra with a header LanguageSwitcher and localStorage persistence, so bilingual content just needed new keys in both locale files - no per-page toggle. ChartDecomp uses inline JS style objects (no CSS modules); matched that. Used returnObjects:true for the benefits array. eslint parse of the edited file passes.</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Overview tab implemented and lints clean. Not yet visually verified in a running build/browser; user should rebuild frontend (npm run build / deploy.sh) and confirm the hover descriptions + pipeline render and switch correctly between EN/VI.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): note docker rebuild step for frontend deploys
Records the deploy gotcha that the screen is served from the baked nginx image,
so host `npm run build` alone does not update it — rebuild the frontend image
(`docker compose ... up -d --build frontend`). Marks the Overview tab DEPLOYED.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -11103,12 +11103,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>The app already has full react-i18next vi/en infra with a header LanguageSwitcher and localStorage persistence, so bilingual content just needed new keys in both locale files - no per-page toggle. ChartDecomp uses inline JS style objects (no CSS modules); matched that. Used returnObjects:true for the benefits array. eslint parse of the edited file passes.</t>
+          <t>The app already has full react-i18next vi/en infra with a header LanguageSwitcher and localStorage persistence, so bilingual content just needed new keys in both locale files - no per-page toggle. ChartDecomp uses inline JS style objects (no CSS modules); matched that. Used returnObjects:true for the benefits array. eslint parse of the edited file passes. DEPLOY GOTCHA: the screen is served by nginx INSIDE the stock_frontend Docker image (baked at image-build time), not from the host build/ folder. A host `npm run build` does NOT update the running screen. To ship frontend changes live: `docker compose -f docker-compose.full-stack.yml up -d --build frontend` (or `./deploy.sh --build`). Confirmed new bundle main.c545210a.js served on :3004 and contains the chart_decomp.overview keys.</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Overview tab implemented and lints clean. Not yet visually verified in a running build/browser; user should rebuild frontend (npm run build / deploy.sh) and confirm the hover descriptions + pipeline render and switch correctly between EN/VI.</t>
+          <t>Overview tab built, tested (4 RTL tests pass), committed (77050294), and DEPLOYED — frontend image rebuilt and stock_frontend recreated; new bundle verified live on :3004. User should hard-refresh (Ctrl+Shift+R) to clear cached old JS. Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(chart-decomp): single combined pattern chart with series toggle
PatternTab single-scale view drew three separate short-axis charts whose
price lines collapsed to near-flat lines (recharts' default 0-anchored Y axis).
Replaced them with one 380px chart on a fitted Y domain (data range ±5%) plus a
"Series" checkbox dropdown (raw, denoised, swing pivots, pattern regions),
matching the project's other multi-series charts. Pivots render via a stroke=none
overlay line so they toggle independently of the denoised line. Legend shows only
visible series; detection report and multi-scale mode unchanged. Adds bilingual
keys (combined_title, series_btn, series_pivots, series_detections, *_short).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11109,6 +11109,33 @@
       <c r="E83" t="inlineStr">
         <is>
           <t>Overview tab built, tested (4 RTL tests pass), committed (77050294), and DEPLOYED — frontend image rebuilt and stock_frontend recreated; new bundle verified live on :3004. User should hard-refresh (Ctrl+Shift+R) to clear cached old JS. Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Pattern Detection tab: merge 3 charts into 1 with series toggle</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Single-scale view of PatternTab (ChartDecomp/index.js) previously rendered three separate stacked charts (Raw vs Denoised, Swing Skeleton, Detected Patterns), each with its own short Y axis anchored at 0 by recharts default -&gt; price series looked like near-flat lines parallel to X. Replaced with ONE 380px-tall combined LineChart on a single Y axis plus a "Series" checkbox dropdown (same UX as UnifiedFinancialChart: button with active-count badge + checkbox list). Toggleable series: raw, denoised, swing pivots (red high / green low dots, rendered via a stroke=none overlay line so they show independently of the denoised line), and pattern regions (ReferenceArea bands, solid=confirmed/dashed=unconfirmed). Added a fitted Y-domain [min-5%, max+5%] computed from raw+denoised values so series fill the height. Legend below shows only visible series; detection report table unchanged; multi-scale mode untouched. New i18n keys (combined_title, series_btn, series_pivots, series_detections, pivots_short, patterns_short) added to both en.json and vi.json.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Root cause of the flat-line look was recharts YAxis default domain starting at 0; explicit fitted domain fixes it. Pivot dots need a backing Line, so used a separate stroke=none Line bound to denoised data with the dot renderer -&gt; pivots toggle works even when the denoised line is off. eslint clean, both locale JSON valid.</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Combined pattern chart built, deployed (frontend image rebuilt, stock_frontend recreated, new bundle main.85b7f5ea.js verified live on :3004 with new keys). User should hard-refresh and re-run a detection to confirm visually. Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(chart-decomp): make Pattern regions toggle reliably show/hide
The Pattern-regions checkbox had no effect because the ReferenceArea bands were
conditionally mounted/unmounted; recharts derives reference-shape state from props
and does not reliably drop those children on unmount, so the bands stayed visible.
Always render the areas now and gate visibility via fill/stroke opacity (a plain
prop update recharts always reflects). Data was fine — the report table reads the
same start_index/end_index fields. Raw/denoised/pivots toggles unchanged.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11136,6 +11136,33 @@
       <c r="E84" t="inlineStr">
         <is>
           <t>Combined pattern chart built, deployed (frontend image rebuilt, stock_frontend recreated, new bundle main.85b7f5ea.js verified live on :3004 with new keys). User should hard-refresh and re-run a detection to confirm visually. Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Fix Pattern regions toggle not hiding/showing on the combined chart</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>In PatternTab combined chart (ChartDecomp/index.js), the Pattern-regions checkbox did nothing because the ReferenceArea bands were conditionally MOUNTED/UNMOUNTED (seriesVis.detections &amp;&amp; dets.map(...)). recharts derives reference-shape state from props and does not reliably drop ReferenceArea children when unmounted, so the bands stayed on screen regardless of the toggle. Fixed by ALWAYS rendering the dets.map ReferenceAreas and gating visibility via opacity instead: fillOpacity = seriesVis.detections ? (confirmed?0.15:0.07) : 0, strokeOpacity = seriesVis.detections ? 0.4 : 0. Data was never the problem (the detection report table reads the same start_index/end_index). Only Pattern-regions visibility behavior changed; raw/denoised/pivots toggles untouched.</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>recharts reliably reflects prop UPDATES on a persistent element but not add/remove of reference children -&gt; prefer opacity toggling over conditional mount for ReferenceArea/ReferenceLine. Applies to any future recharts overlay toggles in this codebase.</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Pattern-regions toggle fixed, eslint clean, frontend image rebuilt + stock_frontend recreated; new bundle main.3d9da498.js live on :3004. User to hard-refresh and verify bands show/hide. Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(portfolio): correct 1000x-inflated total cost in Add Holding
The Add-Holding total-cost preview computed
formatVND(calculateTotalCost(shares, price) * 1000), but formData.price is
already stored in full VND (handleStockSelect converts the thousands-quote at
the boundary) and calculateTotalCost returns shares * price. The extra * 1000
turned 1 share x 12,000 VND into 12,000,000 VND. Removed the stray multiplier;
the current-price field and the save path were already correct.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11190,6 +11190,33 @@
       <c r="E86" t="inlineStr">
         <is>
           <t>Forecast &amp; Back Test fully working. Backend chart-decomp-service rebuilt (off-by-one + winner), frontend rebuilt (bundle main.97063f5d.js). User to hard-refresh, Load Data (2Y), Run Comparison. Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Fix VND total-cost showing 1000x too large in Add Holding</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Portfolio/Holdings.js Add-Holding modal: the Total cost preview computed formatVND(calculateTotalCost(shares, price) * 1000). But formData.price is already stored in FULL VND (handleStockSelect converts the thousands-quote stock.price*1000 at the boundary), and calculateTotalCost returns shares*price (already VND). The extra *1000 made 1 share x 12,000 VND display as 12,000,000 VND. Removed the stray *1000. The Current price field just above (line 373, formatVND(formData.price)) and the save path (handleAddStock -&gt; addStock with parseFloat(formData.price)) were already correct and unchanged.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Unit boundary: stock.price from the options list is a thousands-quote (73.5 = 73,500 VND); the form converts to full VND once on select, so downstream code must NOT re-multiply. The shared formatStockPrice util still *1000s but is correct for its two callers (StockGeneral row.close, Holdings dropdown stock.price) which receive thousands-quotes.</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Total-cost VND fix deployed (frontend bundle main.62ef7c96.js). User to hard-refresh and verify Add Holding total cost. Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(portfolio): stop 1000x-inflating Add Holding prices
Stock options come from the priceboards VN30 endpoint whose matchPrice is
already in full VND (e.g. ACB = 22200), but Holdings assumed a thousands-quote
and multiplied by 1000 twice: the dropdown label via formatStockPrice, and
handleStockSelect storing price * 1000. A real 22,200 ₫ rendered as 22,200,000 ₫
and propagated into the Current price and Total cost fields.

Dropdown now uses formatVND(stock.price); handleStockSelect stores it as-is;
removed the unused formatStockPrice import. Stored unit is unchanged (full VND),
so saved holdings and portfolio totals stay consistent. Verified end-to-end with
Playwright (ACB shows 22.200 ₫ in dropdown, current price, and total cost).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11217,6 +11217,33 @@
       <c r="E87" t="inlineStr">
         <is>
           <t>Total-cost VND fix deployed (frontend bundle main.62ef7c96.js). User to hard-refresh and verify Add Holding total cost. Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Fix Add Holding prices showing 1000x (matchPrice is full VND)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Portfolio/Holdings.js Add-Holding modal showed every price 1000x too large (ACB 22.200.000 instead of 22.200). Root cause: stock options come from the priceboards VN30 endpoint where matchPrice is ALREADY full VND (e.g. ACB=22200.0), but the code assumed a thousands-quote and multiplied by 1000 in two spots: (1) the dropdown label formatStockPrice(stock.price) (the util itself *1000s), and (2) handleStockSelect stored price: stock.price*1000. That inflated input then propagated into Current price and Total cost. Fix: dropdown uses formatVND(stock.price); handleStockSelect stores stock.price as-is; removed the now-unused formatStockPrice import. Stored unit unchanged (full VND) so saved holdings + totals stay consistent. Left the shared formatStockPrice util and its other caller StockGeneral untouched (their data unit not part of this report).</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>The thousands-quote assumption (old comment cited 73.5=73,500) is stale — the priceboards matchPrice now returns full VND, likely from the vnstock 4.x data changes. Verified end-to-end with Playwright on the live app (logged in as tuanph1970, opened Portfolio&gt;Holdings&gt;Add stock, selected ACB): dropdown=22.200, current price=22.200, total cost for 1 share=22.200. Used cached chromium at ~/.cache/ms-playwright/chromium-1208 via executablePath since playwright 1.61 wanted a newer build.</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Add Holding VND fix verified via Playwright + deployed (bundle main.3aa6eab1.js). POSSIBLE FOLLOW-UP: check stocks/StockGeneral.js formatStockPrice(row.close) for the same 1000x issue if its data is now full VND. Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(portfolio): tolerate duplicate default portfolios in get_default_portfolio
GET /portfolios/default (and /watchlist, which depends on it) returned 500
MultipleResultsFound: get_default_portfolio used scalar_one_or_none(), which
throws when a user has more than one is_default=true portfolio (duplicate
defaults from a get-or-create race). That blocked adding any holding at the
first step ("Failed to get portfolio").

Query now orders by created_at/id and limits to 1, returning the oldest default
via scalars().first() — robust to duplicates, fixes both the portfolio and
watchlist 500s. Verified end-to-end: default 200, watchlist 200, buy succeeds.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11244,6 +11244,33 @@
       <c r="E88" t="inlineStr">
         <is>
           <t>Add Holding VND fix verified via Playwright + deployed (bundle main.3aa6eab1.js). POSSIBLE FOLLOW-UP: check stocks/StockGeneral.js formatStockPrice(row.close) for the same 1000x issue if its data is now full VND. Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Fix Add Holding 500: MultipleResultsFound on default portfolio</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Adding a stock failed with "Failed to buy stock: Failed to get portfolio". Root cause: portfolio-service get_default_portfolio (repositories/portfolio_repository.py) used result.scalar_one_or_none(), which RAISES sqlalchemy MultipleResultsFound when a user has more than one is_default=true portfolio (this account had duplicate defaults, likely a get-or-create race). So GET /portfolios/default and GET /watchlist (which calls get_or_create_default_portfolio) both 500d, blocking add-stock at the first step. Fix: query now order_by(created_at asc, id asc).limit(1) + scalars().first() -&gt; deterministically returns the oldest default and never throws on duplicates. One fix covers both the portfolio and watchlist 500s.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>scalar_one_or_none() is a landmine wherever a uniqueness invariant (one default per user) is not actually DB-enforced; prefer limit(1)+first() for "get the one" reads that can have accidental dupes. Verified end-to-end with Playwright on the live account: /portfolios/default 200, /watchlist 200, buy ACB x1 -&gt; 201 at price 22200.0 (VND correct), then deleted the test holding (204) to restore the empty portfolio.</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Default-portfolio 500 fixed; portfolio-service rebuilt + recreated. Duplicate is_default rows still exist in DB (code now tolerates them) - OPTIONAL one-time cleanup to unset extra defaults not yet done. Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(portfolio): heal duplicate default portfolios on startup
Adds an idempotent cleanup in the lifespan (after table creation): for any user
with multiple is_default rows, keep the oldest (MIN(id)) and unset the rest. This
collapses dups left by past get-or-create races so get_default_portfolio has a
single row to return. No-op once clean, so it's safe on every boot.

Verified on the live DB: logged "Cleaned up 1 duplicate default portfolio row(s)";
the account went from two default portfolios to one, /portfolios/default returns 200.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11271,6 +11271,33 @@
       <c r="E89" t="inlineStr">
         <is>
           <t>Default-portfolio 500 fixed; portfolio-service rebuilt + recreated. Duplicate is_default rows still exist in DB (code now tolerates them) - OPTIONAL one-time cleanup to unset extra defaults not yet done. Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>One-time cleanup of duplicate default portfolios</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Added an idempotent startup heal in portfolio-service lifespan (app/main.py), right after Base.metadata.create_all. For any user with multiple is_default=1 portfolios it keeps the oldest (MIN(id) == earliest since id is autoincrement) and unsets is_default on the rest, via a single UPDATE...JOIN (SELECT user_id, MIN(id) keep_id ... GROUP BY user_id HAVING COUNT(*)&gt;1). Logs rowcount when it acts. After the first run no user has dups so it is a no-op on subsequent boots. Complements last session get_default_portfolio limit(1) fix (4c69e9b5): the query is robust to dups AND the data is now actually clean.</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Put it in lifespan (repo self-healing pattern) rather than a manual one-off so it is reproducible and guards against the get-or-create race recurring. Verified on the live DB: startup logged "Cleaned up 1 duplicate default portfolio row(s)"; the test account went from two is_default portfolios (id1,id2) to exactly one (id1 default, id2 not); /portfolios/default returns 200.</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Duplicate-default cleanup deployed + verified (portfolio-service rebuilt). Portfolio default/watchlist/add-holding fully working. Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(prediction): drop all-NaN columns before dropna so simulation can train
_prepare_features ended with a bare df.dropna(). The stock-data-service
history payload returns value/adj_close/change/change_percent as 100% NaN
for some tickers (e.g. ACB), so the unscoped dropna() discarded every row,
leaving 0 training rows and a 422 ("Insufficient training rows before
<start>") on POST /predict/simulation/run. Drop fully-empty columns first
so they neither wipe rows nor leak into _get_feature_columns() as junk
features. Verified: ACB 2023-01-01..2024-01-01 / XGBoost now returns 200.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11298,6 +11298,33 @@
       <c r="E90" t="inlineStr">
         <is>
           <t>Duplicate-default cleanup deployed + verified (portfolio-service rebuilt). Portfolio default/watchlist/add-holding fully working. Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Fix simulation Run 422 (prediction-service)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Root-caused the simulation dashboard 422 (Loi / Server error 422 on POST /predict/simulation/run). It was NOT a request-schema mismatch: SimulationRequest validated fine. The 422 was a SimulationError raised in simulation_service.run_simulation: "Insufficient training rows before &lt;start&gt; (0; need &gt;=30)". Traced into PredictionService._prepare_features (services/prediction-service/app/services/prediction_service.py:74): it ends with df.dropna() (no subset). The stock-data-service /stocks/{sym}/history payload returns value/adj_close/change/change_percent as 100% NaN for ACB (523/523), so the unscoped dropna() discarded EVERY row -&gt; 0 train rows. Fix: added df = df.dropna(axis=1, how="all") just before the row-wise dropna() at prediction_service.py:122, dropping fully-empty columns so they neither wipe rows nor leak into _get_feature_columns() as junk features.</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>The data-quality bug is upstream in stock-data-service (those 4 raw OHLCV-adjacent columns come back all-null), but fixing _prepare_features to be robust to all-NaN columns is the correct general fix and also benefits the production train/predict path which shares this builder. Verified end-to-end: feature prep now keeps 473 rows (225 pre-start train rows) for ACB 2021-11..2024-01; POST /simulation/run for ACB 2023-01-01..2024-01-01 / XGBoost returns HTTP 200 with metrics, accuracy, 248 time-series points, 2 transactions.</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Backend fix applied to source + hot-loaded into running stock_prediction_service (docker cp + restart) so it works in the live UI now. Needs ./deploy.sh --build (or rebuild prediction-service image) to bake it in permanently. Consider a follow-up to fix stock-data-service so value/adj_close/change/change_percent are populated.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(predict,auth): real walk-forward backtest + send token in /verify body
Backtest "Run backtest" returned 404: PredictionService.backtest only
summarized previously-stored live predictions, which never exist for a
fresh request, so it returned None and the route raised 404. Rewrite it
as a walk-forward backtest that re-runs the active model over the
historical window (causal per-step features, direction hit-rate + MAE +
RMSE + volatility-based confidence). Update unit tests to the new path
and soften the route's 404 message.

Auth /verify returned 422 on every page load: the frontend posted the
JWT only in the Authorization header with no body, but the backend's
TokenVerify schema requires the token in the JSON body. Send
{ token } in the request body.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11325,6 +11325,60 @@
       <c r="E91" t="inlineStr">
         <is>
           <t>Backend fix applied to source + hot-loaded into running stock_prediction_service (docker cp + restart) so it works in the live UI now. Needs ./deploy.sh --build (or rebuild prediction-service image) to bake it in permanently. Consider a follow-up to fix stock-data-service so value/adj_close/change/change_percent are populated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Fix Backtest screen 404 (prediction-service)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Root-caused the Backtest page error (POST /stock_helper/api/v2/predict/backtest -&gt; 404). Traefik routing was fine (full-stack compose routes /predict). The 404 was business-logic: PredictionService.backtest (services/prediction-service/app/services/prediction_service.py:402) only *summarized* previously-stored live predictions via repo.get_predictions(); a fresh "Run backtest" click for any symbol/period never run live had zero stored rows -&gt; returned None -&gt; route raised 404. Rewrote backtest() as a real walk-forward backtest: fetch history (window + 120d warm-up), build causal features via _prepare_features, restrict to [start,end], load/train the active model, predict next-day close per windowed day, score direction hit-rate + MAE + RMSE + a volatility-based confidence proxy. Updated the 2 unit tests in tests/test_prediction_service.py to cover the new path; softened the route 404 message in routes.py.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>The old backtest was effectively a stub keyed to live-stored predictions, so the feature could only ever 404 in normal use. New impl reuses the same _fetch_historical_data + _prepare_features path as predict(); per-step features are causal but the model may have trained on overlapping data, so results are indicative not strictly leakage-free (noted in docstring). All 20 prediction_service unit tests pass.</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Fix applied to source, prediction-service image rebuilt, container recreated on the live stack (port 18004). Verified the route is reached (401 without token = routed+live; logged-in UI supplies the token). Next: have the user click Run backtest in the UI to confirm 200 with metrics. Note: a separate 422 on /auth/verify was visible in the console but is unrelated to this fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Fix /auth/verify 422 (frontend)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Root-caused the console 422 on POST /stock_helper/api/v2/auth/verify. Contract mismatch: auth-service verify_token expects the TokenVerify body {"token": "..."} (schemas.py:87, token: str required), but authService.checkAuth in stock_react_javascript/.../src/services/api.js:174 called fetch(AUTH_VERIFY, {method:POST, headers:getAuthHeaders()}) with the JWT only in the Authorization header and NO body -&gt; FastAPI reported the required token field missing -&gt; 422. Fix: added body: JSON.stringify({ token }) to the verify fetch (token already read at api.js:166).</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Verified against the live backend on :18004: POST /auth/verify with no body -&gt; 422 (repro); with {"token":"..."} body -&gt; 200 {valid:false} for an invalid token (would be valid:true for a real one). The endpoint validates via the body, not the header.</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Frontend fix applied; frontend Docker image rebuilt and stock_frontend container recreated on the live stack (:3004, healthy) so the running screen no longer fires the 422 on load. Both this session fixes (backtest 404 + auth/verify 422) are now baked into images.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(chart-decomp): polish Pattern Detection tab UX
- Add hover info tooltips (EN+VI) for the Multi-scale (nested),
  Scales (k_drop) and Denoise k_drop labels via a new InfoTip
  component; help text added to en.json + vi.json.
- Format Y axis to one decimal (e.g. 21.2) and widen the axis so
  labels no longer clip/show abnormal cut-off values.
- Show dates on the X axis as dd/mm/yy with ~one tick per 3 months;
  thread trading dates InputPanel -> ChartDecompPage -> PatternTab
  (demo series with no dates falls back to the numeric index).
- Hide detections scoring < 70% from both the report tables and the
  chart regions, in single-scale and multi-scale modes.
- Box each detected region's ReferenceArea to the data min/max Y over
  [start_index, end_index] instead of spanning the full chart height.

Also updates ROADMAP.xlsx (Sessions Log + Feature Inventory).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -4524,7 +4524,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Panel1 raw/denoised, Panel2 swing skeleton H/L dots, Panel3 ReferenceArea per detection. FR-VIZ-2 report table: pattern/start/end/score/confirmed/null-pct95.</t>
+          <t>Panel1 raw/denoised, Panel2 swing skeleton H/L dots, Panel3 ReferenceArea per detection. FR-VIZ-2 report table: pattern/start/end/score/confirmed/null-pct95. | 2026-06-24 UX polish: i18n hover tips (multi-scale/k_drop), Y axis 1-decimal (no clipping), X axis dates dd/mm/yy ~quarterly ticks, hide detections &lt;70% from table+regions, region rectangles boxed to data min/max Y over [start,end].</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11406,6 +11406,33 @@
       <c r="E94" t="inlineStr">
         <is>
           <t>Frontend rebuilt + stock_frontend recreated (:3004) with the display fix in the previous turn; the test-only changes do not affect the bundle so the running UI is already correct. Ready to commit; deploy-interactive.sh left uncommitted (pre-existing, unrelated).</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>ChartDecomp Pattern Detection — UX polish (tooltips, axes, region boxes, score filter)</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Improved the Pattern Detection tab (src/components/Pages/ChartDecomp/index.js + i18n). (1) Added hoverable info (i) tooltips next to the Multi-scale (nested), Scales (k_drop) and Denoise k_drop labels via a new InfoTip component; help text added to en.json + vi.json (ms_toggle_tip, ms_scales_tip, k_drop_tip). (2) Y axis now formats to 1 decimal (toFixed(1), e.g. 21.2) with width 52 so labels no longer clip — fixes the abnormal/cut-off values. (3) X axis now shows dates dd/mm/yy with ~one tick per 3 months (quarterlyTickIndices picks the first index of each new quarter); Tooltip label formatted too. Trading dates are threaded InputPanel-&gt;ChartDecompPage-&gt;PatternTab (new dates prop/state); demo series (no dates) falls back to numeric index. (4) Detections with score &lt; 70% are filtered out of both the report tables and the chart regions, in single-scale and multi-scale modes (MIN_PATTERN_SCORE=0.70). (5) Each detected region ReferenceArea is now boxed by y1/y2 = data min/max over [start_index,end_index] (new rangeYBounds helper) instead of spanning full height; single-scale bounds raw+denoised, multi-scale bounds the detection scale series (fallback coarsest/raw).</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>series passed to PatternTab was prices-only; dates were dropped at load. Fixed by pairing price+date in InputPanel before the null-filter so they cannot desync. StockPriceResponse exposes a date field (YYYY-MM-DD). recharts category XAxis accepts an explicit ticks subset of the data indices; ReferenceArea positions by axis value regardless of ticks.</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>All changes applied to source; CI=false npm run build compiles successfully (+2.29kB). NOT yet live on the running screen — frontend Docker image must be rebuilt (./deploy.sh --build) per project memory; host npm run build alone does not update the container. Changes not yet committed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(chart-decomp): visible grid + dated start/end in Pattern Detection
- Make the Pattern Detection chart grids clearly visible: gray-300
  (#cbd5e1) dashed grid with explicit horizontal+vertical lines,
  replacing the near-invisible gray-200 grid. Other tabs unchanged.
- Report-table Start/End columns now render as dd/mm/yyyy dates
  (fmtDDMMYYYY + idxDate using the dates prop) instead of raw indices;
  falls back to the index for the demo series with no dates.

Also updates ROADMAP.xlsx (Sessions Log).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11433,6 +11433,33 @@
       <c r="E95" t="inlineStr">
         <is>
           <t>All changes applied to source; CI=false npm run build compiles successfully (+2.29kB). NOT yet live on the running screen — frontend Docker image must be rebuilt (./deploy.sh --build) per project memory; host npm run build alone does not update the container. Changes not yet committed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>ChartDecomp Pattern Detection — visible grid + dated start/end columns</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Two follow-up tweaks to the Pattern Detection tab (ChartDecomp/index.js). (1) Made the chart grid clearly visible: the 3 pattern charts now use CartesianGrid stroke #cbd5e1 (gray-300) dashed 3 3 with explicit horizontal+vertical, replacing the near-invisible #e5e7eb grid. Other tabs unchanged. (2) Report table Start/End columns now show full dates dd/mm/yyyy (new fmtDDMMYYYY helper + idxDate formatter using the dates prop) instead of raw integer indices; falls back to the index for the demo series with no dates.</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Existing grid was present but #e5e7eb was too faint to read as a grid; bumping to gray-300 + forcing vertical lines fixes the perceived missing grid. Table dates reuse the same dates[] already threaded for the X axis.</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Built + frontend Docker image rebuilt + stock_frontend recreated (:3004, healthy, bundle main.05b58ae1.js); #cbd5e1 and vertical-grid confirmed in served JS. Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(chart-decomp): darker grid (slate-400) for visibility on white
Pattern Detection chart grid lines were too faint on a white
background (#cbd5e1); switch to #94a3b8 so the grid reads clearly
without overpowering the data lines.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11460,6 +11460,33 @@
       <c r="E96" t="inlineStr">
         <is>
           <t>Built + frontend Docker image rebuilt + stock_frontend recreated (:3004, healthy, bundle main.05b58ae1.js); #cbd5e1 and vertical-grid confirmed in served JS. Ready to commit/push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>ChartDecomp Pattern Detection — darker grid for visibility</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Grid lines on the 3 pattern charts were too faint on white (#cbd5e1 slate-300); bumped to #94a3b8 (slate-400). Frontend Docker image rebuilt + stock_frontend force-recreated (:3004 healthy, bundle main.b7d5535b.js); #94a3b8 confirmed in served JS.</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>User feedback: grid+dates render correctly but grid color was hard to see on white background.</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Deployed and verified live. Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(vol-forecast): dual independent Y axes on OOS log-RV chart
The actual log-RV (a 1-day proxy) spikes from ~-5 to ~-27 while the
HAR/VMD-HAR forecasts stay smooth near the mean, so on one shared Y
axis the forecasts looked flat. Split the comparison chart into
independent left/right axes (both in log-RV units): actual on the
left (full range), forecasts on the right (auto-zoomed to their own
range) so their movement is visible. Adds axis labels, a dual-axis
caption, colored ticks, and a clearer grid. New i18n keys in en+vi.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11487,6 +11487,33 @@
       <c r="E97" t="inlineStr">
         <is>
           <t>Deployed and verified live. Ready to commit/push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Vol-Forecast — dual-axis OOS log-RV chart + explained metrics</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>User asked why the HAR/VMD-HAR forecast lines look flat vs the actual on the OOS chart. Root cause: the log-RV target is a 1-day proxy log(r^2+1e-12) so actual swings ~-5..-27 (spikes to -27 on near-zero-return days) while HAR/VMD-HAR forecast a smooth level near the mean; on one shared Y axis the forecasts are crushed flat. Fix (ComparePanel in VolForecastPage.js): split into independent left/right Y axes (both log-RV units) — actual on LEFT (full range), HAR+VMD-HAR on RIGHT auto-zoomed via padDomain(); added axis labels + a dual_axis_hint caption + colored ticks; also upgraded the chart grid to #94a3b8 dashed h+v. New i18n keys dual_axis_hint/axis_actual/axis_pred in en+vi. Verified by replaying the exact pipeline on REAL VCB data (gateway /stocks/VCB/history -&gt; log-RV -&gt; /forecast/compare): HAR rmse5.49 mae3.33 r2~0 qlike22.6, VMD-HAR worse (winner=HAR, DM=-2.77) — matches the users screenshot numbers.</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Vol-Forecast loads REAL prices via companyService.getCompanyCharts (history endpoint); only the green Demo button is synthetic. Metrics: RMSE/MAE in log-RV units, R2 vs predicting the mean (~0 = no skill, negative = worse than mean), QLIKE=mean(var_true/var_pred - log(ratio) -1) on the variance scale. The R2 delta 83625% is an artifact of dividing by HAR R2 ~0.0003 (near-zero baseline). The 1-day RV proxy is inherently near-unpredictable; this is expected, not a bug.</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + stock_frontend recreated (:3004 healthy, bundle main.b02449c4.js); dual-axis confirmed in served JS. Reproduced real-data preview PNG. Ready to commit/push. Possible follow-up: the noisy 1-day RV proxy could be replaced with a rolling/Parkinson RV for more meaningful forecasts.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(vol-forecast): rolling Parkinson RV target + Introduction tab
- Replace the noisy 1-day close-to-close RV proxy with a rolling
  Parkinson high-low realized-variance target (dailyParkinsonVar +
  rollingParkinsonLogRV). DataPanel now passes OHLC; a configurable
  rolling window (default 5) drives a useMemo-derived log-RV. On real
  VCB data this lifts HAR out-of-sample R2 from ~0.00 to ~0.90.
- Add a bilingual Introduction tab (Definition / Goal / How to achieve)
  with a tab bar (Introduction | Forecast & Backtest); full EN + VI
  i18n under vol_forecast.intro.* and config.rv_*.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11514,6 +11514,33 @@
       <c r="E98" t="inlineStr">
         <is>
           <t>Frontend rebuilt + stock_frontend recreated (:3004 healthy, bundle main.b02449c4.js); dual-axis confirmed in served JS. Reproduced real-data preview PNG. Ready to commit/push. Possible follow-up: the noisy 1-day RV proxy could be replaced with a rolling/Parkinson RV for more meaningful forecasts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Vol-Forecast — rolling Parkinson RV target + bilingual Introduction tab</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>(1) Replaced the noisy 1-day close-to-close RV proxy log(r^2+1e-12) with a rolling Parkinson high-low realized-variance target in VolForecastPage.js: new dailyParkinsonVar (sigma2=(ln(H/L))^2/(4ln2), falls back to squared close-to-close when H/L missing) + rollingParkinsonLogRV (expanding-&gt;rolling mean, then log). DataPanel now extracts OHLC (high/low/close) and passes {prices,highs,lows}; demo synthesizes a high/low band. logRV is now a useMemo over (prices,bars,rv_window). Added a Realized-variance config section with rv_window (default 5) + hint. (2) Added an Introduction tab (tab bar: Introduction | Forecast &amp; Backtest, default=Introduction) with Definition / Goal / How-to-achieve (6 numbered steps) via new IntroTab; full EN+VI i18n under vol_forecast.intro.* plus config.rv_* keys and an updated page_subtitle.</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Verified the RV change on REAL VCB data via the gateway pipeline: rolling Parkinson w=5 lifts HAR R2 from ~0.0000 to 0.9001 (RMSE 5.49-&gt;0.30, QLIKE 22.6-&gt;0.05); w=10 R2=0.956. log_rv range tightens from -27.6..-5.3 to -11.7..-6.0 (no more spurious -27 spikes on near-zero-return days). VMD-HAR still loses to HAR (winner=HAR, honest C4 benchmark). The high R2 reflects the smoother, autocorrelated rolling target - standard for RV/HAR forecasting. i18n arrays use returnObjects:true for how_steps.</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + stock_frontend recreated (:3004 healthy, bundle main.cdffb195.js); Parkinson helper + Intro (EN escaped-VI) + rv config all confirmed in served JS. Reproduced real-data dual-axis chart (forecasts now track actual). Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(vol-forecast): series toggle dropdowns + merged backtest chart
- Forecast OOS chart: add a reusable SeriesToggle checkbox dropdown to
  show/hide actual/HAR/VMD-HAR (the two forecasts overlap closely under
  the Parkinson RV target, so one looked hidden); grid confirmed.
- Backtest: merge the four separate charts into one ComposedChart with
  dual independent Y axes (left = Net P&L + Buy&Hold + Drawdown; right =
  Position + Turnover), grid, padded domains, and the same toggle.
- Remove now-unused recharts imports; new i18n keys in en + vi.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11541,6 +11541,33 @@
       <c r="E99" t="inlineStr">
         <is>
           <t>Frontend rebuilt + stock_frontend recreated (:3004 healthy, bundle main.cdffb195.js); Parkinson helper + Intro (EN escaped-VI) + rv config all confirmed in served JS. Reproduced real-data dual-axis chart (forecasts now track actual). Ready to commit/push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Vol-Forecast — series toggle dropdowns + merged backtest chart</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>(1) Forecast OOS chart (ComparePanel): added a reusable SeriesToggle checkbox-dropdown to show/hide actual/HAR/VMD-HAR (HAR &amp; VMD-HAR overlap closely under Parkinson RV, so one looked hidden); grid was already present (#94a3b8 h+v) and confirmed. useState moved above the early return to satisfy rules-of-hooks. (2) Backtest (BacktestPanel): replaced the 4 separate charts (equity/drawdown/collapsible position/turnover) with ONE merged ComposedChart — dual independent Y axes (left = Net P&amp;L + Buy&amp;Hold + Drawdown; right = Position w[t] + Turnover), #94a3b8 grid, padded auto-domains that ignore hidden series, and the same SeriesToggle. Removed showPos/showTurn state and now-unused recharts imports (AreaChart/Area/Bar). New i18n: compare.series_btn, backtest.combined_title/dual_axis_hint/axis_pnl/axis_exposure (en+vi).</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Verified the merged backtest layout on REAL VCB data (Parkinson compare -&gt; /backtest/vol-target: 529 aligned points/series; metrics ann_ret 3.3%, sharpe 0.17, maxdd 20%, avg_lev 1.01). Reused buildCumPnl/buildDrawdown shapes; positions/turnover aligned by index with ?. guards. SeriesToggle is shared by both charts.</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + stock_frontend recreated (:3004 healthy, bundle main.dbf2d13d.js); SeriesToggle + axis_exposure confirmed in served JS; real-data preview rendered. Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(journal): add Overview submenu with guide + pipeline diagram
New Trade Journal > Overview screen (mirrors Decision Helper's General
View): a static why-it-matters paragraph, a benefits grid, and a
6-stage journaling pipeline (Plan -> Execute -> Log -> Reflect ->
Review -> Improve) with a continuous-improvement loop. Wired the
route and a sidebar entry; full EN + VI i18n. Relabelled the existing
journal_dashboard from "Overview" to "Dashboard" to avoid a duplicate
label (it is a stats dashboard).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11568,6 +11568,33 @@
       <c r="E100" t="inlineStr">
         <is>
           <t>Frontend rebuilt + stock_frontend recreated (:3004 healthy, bundle main.dbf2d13d.js); SeriesToggle + axis_exposure confirmed in served JS; real-data preview rendered. Ready to commit/push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Trade Journal — new Overview submenu (guide + pipeline diagram)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Added a new Overview submenu under Trade Journal (first item), mirroring Decision Helper General View. New component src/components/Pages/Journal/JournalOverview.js: page header + a static why-it-matters paragraph + a benefits grid (6 items) + a 6-stage journaling pipeline diagram (Plan-&gt;Execute-&gt;Log-&gt;Reflect-&gt;Review-&gt;Improve) reusing the Box/Arrow/SectionTitle visual primitives, plus a continuous-improvement loop pill and a legend. Wired route /journal-overview in MainLayout.js and a journal-overview submenu entry in Sidebar.js. Full EN+VI i18n under journal.overview.* (benefits uses returnObjects array). Renamed the existing sidebar label journal_dashboard from Overview-&gt;Dashboard (EN) / Tong quan-&gt;Bang thong ke (VI) to avoid a duplicate Overview label, and added sidebar.journal_overview = Overview / Tong quan.</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>The existing journal_dashboard was already labelled Overview but is actually a stats dashboard; relabelled it to Dashboard so the new guide can own the Overview name. Reused the DecisionHelperOverview primitive components (copied locally, not exported). i18n VI is unicode-escaped in the bundle (normal).</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + stock_frontend recreated (:3004 healthy, bundle main.f71de320.js); route + EN/VI content + pipeline confirmed in served JS. Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): content-area theme derived from AIKnow reference
Add src/theme.css with design tokens + base styling for text fields,
dropdowns, buttons and tables, derived from the AIKnow reference UI
(Inter, primary #4192f7, border #d0d5dd, 8px input radius, etc).

Scoped to .app-theme on the .page-content area only: the left sidebar
and top header (outside .page-content) are untouched, and the Price
Board route omits .app-theme so it stays exactly as-is. Data-grid cell
text color is intentionally left unchanged. Only native/class-based
(non-inline) elements are affected.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11595,6 +11595,33 @@
       <c r="E101" t="inlineStr">
         <is>
           <t>Frontend rebuilt + stock_frontend recreated (:3004 healthy, bundle main.f71de320.js); route + EN/VI content + pipeline confirmed in served JS. Ready to commit/push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Global content theme from AIKnow reference (scoped, sidebar+priceboard excluded)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Used Playwright (python, headed via DISPLAY=:0) to inspect the reference app http://aiknow-dev.technica.vn (login tuongnm/123456) Documents screen and extract computed styles from the live DOM. Derived design tokens: Inter font; primary #4192f7; text #344054; heading #101828; muted #7e8083; input border #d0d5dd radius 8px; general border #e4e7ec; inputs 16px/height44/padding 9px 14px; buttons radius 4px font 16/600. Created src/theme.css (scoped under .app-theme): CSS vars + Inter @import + base styling for input/textarea/select (+chevron, focus ring) , buttons (font/radius + .btn-primary/.btn-secondary helpers), tables (borders+padding+font, NO cell text color per request), headings. Imported in index.js. MainLayout: added useLocation; &lt;main className=page-content {app-theme unless /priceboard}&gt;. Sidebar+header are outside .page-content so untouched; Price Board route omits .app-theme so unchanged.</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>User chose Global base theme scope: only restyles native/class-based (non-inline) elements; inline-styled charts/dashboards keep their look. Constraints: do not change the left sidebar (only content area) and leave Price Board exactly as-is. getComputedStyle reads the live DOM = the reliable source (vs parsing raw bootstrap css). Inter was NOT previously loaded; theme.css now @imports it.</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + stock_frontend recreated (:3004 healthy, css bundle main.6496ad19.css; theme markers + priceboard exclusion confirmed). Ready to commit/push. User may fine-tune sizes (16px/44px) after visual review.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ui): force-override content theme so it actually applies
The base theme was outranked by the app's inline styles and per-page
CSS (e.g. oversized grid headers). Switch theme.css to use !important
on font/size/border/radius/padding for inputs, selects, textareas,
table th/td and headings, scoped to .app-theme. Grid headers/cells are
forced to 13px (fixes big headers); inputs 15px with an 8px radius and
focus ring. Sidebar, header, Price Board and grid text color remain
untouched.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11622,6 +11622,33 @@
       <c r="E102" t="inlineStr">
         <is>
           <t>Frontend rebuilt + stock_frontend recreated (:3004 healthy, css bundle main.6496ad19.css; theme markers + priceboard exclusion confirmed). Ready to commit/push. User may fine-tune sizes (16px/44px) after visual review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Content theme escalated to force-override (visible app-wide)</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Base theme was barely visible because the app uses heavy inline styles + per-page CSS classes that outrank a low-specificity global stylesheet (e.g. big grid headers). Per user choice, switched src/theme.css to FORCE-OVERRIDE: !important on font-family/size/border/radius/padding for inputs, textareas, selects (+chevron, focus ring), table th/td, and headings; inputs 15px / min-height 42px / 8px radius; table th &amp; td forced to 13px to shrink oversized grid headers; buttons get Inter font (+ .btn-primary/.btn-secondary helpers). Still scoped to .app-theme only; grid cell TEXT COLOR never set; buttons border-radius left non-important so pill/icon buttons survive.</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Confirmed Docker WAS rebuilt earlier (git push does not rebuild). getComputedStyle/base-theme could not override inline+class styles; only !important within .app-theme does. Sidebar/header are outside .page-content; Price Board route omits .app-theme.</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + recreated (:3004 healthy, css bundle main.fd6b6318.css, force rules live). Ready to commit/push. User to review; sizes (15px inputs / 13px grid) easy to fine-tune.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): centralize retheme — flip design tokens to AIKnow in .app-theme
The cream + Instrument-Serif identity comes from CSS variables in
index.css. Re-point those tokens (--paper/--panel/--line, --ink2/3,
--font-sans/serif/mono) to the AIKnow palette inside .app-theme so every
content page rethemes from one place: white surfaces, cool-gray borders,
Inter fonts. Base --ink kept so data-grid text color is unchanged.
Sidebar/header and Price Board keep the original tokens; special screens
can override locally.

Verified: content bg cream (230,227,218) -> white (255,255,255), fonts -> Inter.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:F104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11649,6 +11649,33 @@
       <c r="E103" t="inlineStr">
         <is>
           <t>Frontend rebuilt + recreated (:3004 healthy, css bundle main.fd6b6318.css, force rules live). Ready to commit/push. User to review; sizes (15px inputs / 13px grid) easy to fine-tune.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Centralized retheme: flip design tokens to AIKnow inside .app-theme</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>The app identity (cream + Instrument-Serif + mono) is driven by CSS variables in index.css (--paper, --panel, --line, --font-sans/serif/mono, --ink2/3). Re-pointed those tokens to the AIKnow palette INSIDE .app-theme (theme.css): --paper/--panel #fff, --line #e4e7ec, --ink2/3 cool grays, all three font vars -&gt; Inter, plus background:#fff!important. Base --ink kept so data-grid text color is unchanged. Sidebar/header (outside .page-content) and Price Board (omits .app-theme) keep original tokens; special screens can override locally.</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Verified via Playwright login (tuanph1970@gmail.com): computed main.page-content.app-theme bg=rgb(255,255,255), font resolves to Inter, --paper=#fff, --font-serif=Inter. Pixel sample of dashboard bg before=(230,227,218 cream) -&gt; after=(255,255,255 white). @import Inter is valid (after @charset) and index.html already loads Geist/Instrument; theme adds Inter. Remaining AIKnow gap = accent colors (green/black vs blue) which are inline/semantic -&gt; per-screen.</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + recreated (:3004 healthy, css main.149baa29.css). Retheme confirmed working (white+Inter). Ready to commit/push. Next optional: per-screen blue accent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): blue accent (#4192f7) for content-area primary buttons
Re-point the centralized --ui-primary token to the AIKnow blue inside
.app-theme, and map the legacy dark "primary" buttons (.dashboard-primary-btn,
.btn-submit, .add-new-button, [class*=primary-btn]) to it so the Dashboard
"+ Add stock" and similar near-black buttons become blue. Semantic green/red
P&L colors are left unchanged.

Verified: + Add stock button now rgb(65,146,247) = #4192f7.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11676,6 +11676,33 @@
       <c r="E104" t="inlineStr">
         <is>
           <t>Frontend rebuilt + recreated (:3004 healthy, css main.149baa29.css). Retheme confirmed working (white+Inter). Ready to commit/push. Next optional: per-screen blue accent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Blue accent (AIKnow #4192f7) for content-area primary buttons</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Discovered theme-ui.css already has a centralized blue button system (--ui-primary #1677ff on :root, scoped .page-content). In theme.css .app-theme: (1) re-pointed --ui-primary/-hover/-active to AIKnow #4192f7/#5a9ef8/#2f7fe0 (works because .app-theme on &lt;main&gt; is a closer ancestor than :root for inherited custom props); (2) extended the primary-button rule to also recolor the LEGACY dark buttons that use var(--ink) — .dashboard-primary-btn (Dashboard +Add stock), .btn-submit, .add-new-button, [class*=primary-btn] — to var(--c-primary) with white text. Semantic --pos/--neg (green/red P&amp;L) left unchanged.</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Verified: Dashboard +Add stock button pixel was black before, now (65,146,247)=#4192f7; day-change % stays green. Custom-property inheritance: nearest ancestor that defines the var wins for descendants regardless of :root specificity, so .app-theme override beats theme-ui :root.</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + recreated (:3004 healthy). Blue accent live + verified. Ready to commit/push. Inline-accent pages (ChartDecomp/VolForecast indigo) remain per-screen if wanted.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): sentence-case labels — remove ALL-CAPS in content area + header
- Turn off text-transform:uppercase inside .app-theme so labels render in
  their natural sentence case (Total value, Day change, Symbol, ...).
- Header chrome: .header-meta uppercase->none; i18n UPDATED->Updated,
  MARKET OPEN/CLOSED -> Market open/closed (en + vi).
- Fix the Dashboard wordmark "Dash board" -> "Dashboard" (emphasis was
  splitting the single word).
- stat_pnl "Profit / Loss" -> "Profit / loss". Acronyms (QLIKE, VMD-HAR,
  SMA, EPS) are literal in the strings and unaffected.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11703,6 +11703,33 @@
       <c r="E105" t="inlineStr">
         <is>
           <t>Frontend rebuilt + recreated (:3004 healthy). Blue accent live + verified. Ready to commit/push. Inline-accent pages (ChartDecomp/VolForecast indigo) remain per-screen if wanted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Sentence-case labels: remove ALL-CAPS in content + header wordmark</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Most caps came from CSS text-transform:uppercase over already sentence-case strings. theme.css: .app-theme,.app-theme * {text-transform:none!important} so labels show natural case. Header chrome fixed directly: layout.css .header-meta uppercase-&gt;none; i18n UPDATED-&gt;Updated, MARKET OPEN/CLOSED-&gt;Market open/closed en + Thi truong mo/dong, Cap nhat vi. Dashboard wordmark Dash board-&gt;Dashboard via page_titles.dashboard.emphasis board-&gt;Dashboard. stat_pnl Profit / Loss -&gt; Profit / loss. Acronyms QLIKE/VMD-HAR/SMA/EPS are literal and unaffected.</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>~31 uppercase rules across 12 css files; disabling transform was enough. Sidebar/Price Board still excluded. Remaining Title-Case source strings on other screens would need a per-string sweep for full sentence case.</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Verified on Dashboard: header Updated.. Market open.. Dashboard; content labels sentence case; +Add stock still blue. Frontend rebuilt + recreated :3004. Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): unify data grids to the AIKnow look; Price Board excluded
Make theme-ui.css the single source of truth for grids: align the row
divider to #e4e7ec and the header to 12px (matching the AIKnow Material
table), and remove the conflicting .app-theme table th/td !important
rules from theme.css that were forcing 13px.

Result: all themed grids share one clean white look (subtle gray header,
horizontal #e4e7ec dividers, no zebra, Inter) with semantic cell text
colors preserved. The Price Board (.services .custom-table) stays its
dark, market-color-coded terminal via the existing hard exclusion.

Verified: Watchlist grid restyled; Price Board unchanged (blue up / red down).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11730,6 +11730,33 @@
       <c r="E106" t="inlineStr">
         <is>
           <t>Verified on Dashboard: header Updated.. Market open.. Dashboard; content labels sentence case; +Add stock still blue. Frontend rebuilt + recreated :3004. Ready to commit/push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Unify all data grids to the AIKnow look (Price Board excluded)</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Inspected AIKnow /documents grid via Playwright (Angular Material table): cells 14px #344054, header 12px wt500, row divider 1px #e4e7ec, padding ~12px, white no-zebra. Found the app already has a centralized grid theme in theme-ui.css (.page-content table/th/td + .custom-header/.custom-row + .rdt_* react-data-table) that never sets cell color. Made it the single source: removed the conflicting .app-theme table th/td !important block from theme.css (was forcing 13px); aligned theme-ui --ui-split #f0f0f0 -&gt; #e4e7ec and th font-size -&gt; 12px with secondary color. Result: unified white grid, gray subtle header, e4e7ec horizontal dividers, no zebra, Inter, semantic cell colors preserved.</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Price Board is hard-excluded: it is wrapped in .services with table.custom-table, and theme-ui re-asserts dark #0F0F0F cells / #333 borders / 0.75rem at higher specificity; plus the grid theme never sets cell text color so blue=up/red=down market semantics survive. Verified by screenshots: Watchlist grid = AIKnow style; Price Board = unchanged dark terminal with colors.</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + recreated (:3004 healthy). Verified Watchlist (themed) + Price Board (untouched). Coverage: HTML tables, .custom-header/.custom-row, react-data-table. A few div grids with bespoke classes (e.g. Stocks .results-header) may need per-screen coverage. Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): simplify Stocks grid headers + add row dividers
The Stocks screener/industry/stocklist tables used per-column gradient
headers (purple/blue/orange/red...) and zebra rows defined with
!important in StockComponents.css. Append a unified override (.stocks-table
thead th / th[class*=th-]) -> one subtle gray header (#fafafa, #475467,
12px, no gradient), clean #e4e7ec row dividers on every td, and white
non-zebra rows. Semantic up/down cell colors are preserved; the Price
Board (.custom-table) is unaffected.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11757,6 +11757,33 @@
       <c r="E107" t="inlineStr">
         <is>
           <t>Frontend rebuilt + recreated (:3004 healthy). Verified Watchlist (themed) + Price Board (untouched). Coverage: HTML tables, .custom-header/.custom-row, react-data-table. A few div grids with bespoke classes (e.g. Stocks .results-header) may need per-screen coverage. Ready to commit/push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Stocks submenus: simplify colourful grid headers + add row lines</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>The Stocks pages (screener/byindustry/stocklist) tables use .stocks-table + per-column gradient headers (.th-symbol purple, .th-price orange, .th-change red, etc.) defined with !important in stocks/StockComponents.css, plus zebra rows. They sit inside .services so theme-ui did not normalize them. Appended a unified override at the END of StockComponents.css: .stocks-table thead th and .stocks-table th[class*=th-] -&gt; subtle #fafafa header, #475467 text, 12px, no gradient/!important (specificity 0,2,1 beats the 0,2,0 colour rules and wins by source order); .stocks-table td border-bottom 1px #e4e7ec (row lines); row-even/odd -&gt; white (no zebra). Semantic cell colours (up/down) untouched. Price Board uses .custom-table not .stocks-table so unaffected.</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Verified Stock list grid: single gray header (was rainbow per-column), clean e4e7ec row dividers, white rows, blue links, amber exchange badge kept. byindustry/stockscreener share .stocks-table so same fix applies once their data shows. Note: the green .screen-button (Search) is still off-brand green; can blue-ify later if wanted.</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + recreated (:3004 healthy). Stock list verified. Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): unify Stocks action buttons to AIKnow blue
Make .search-button (green), .analysis-button (teal) and .screen-button
(blue gradient) a solid #4192f7 with white text and #2f7fe0 hover, for
consistency with the rest of the app. Neutral gray .details-button stays
as the secondary style.

Verified: Stock list Search button is now rgb(65,146,247) = #4192f7.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11784,6 +11784,33 @@
       <c r="E108" t="inlineStr">
         <is>
           <t>Frontend rebuilt + recreated (:3004 healthy). Stock list verified. Ready to commit/push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Stocks action buttons -&gt; AIKnow blue for consistency</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Unified the Stocks primary action buttons to #4192f7 in StockComponents.css: .search-button (was green gradient), .analysis-button (was teal #17a2b8), .screen-button (was blue gradient) -&gt; solid blue, white text, hover #2f7fe0, no gradient. Neutral gray .details-button kept as secondary; pagination unchanged.</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Verified Stock list Search button pixel = (65,146,247) = #4192f7. Grid header simplification + row dividers from prior commit still in place.</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + recreated (:3004 healthy). Verified. Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): simplify Portfolio grids (Holdings, Alerts) to AIKnow look
Holdings (.portfolio-table) and Alerts (.alerts-table) had gradient
headers, zebra rows, scale-hover and gradient-text stat values. Append
unified overrides: subtle gray header (#fafafa / #475467 / 12px), clean
#e4e7ec row dividers, white non-zebra rows, calm hover, 13px cells. The
decorative gradient-text stat values become solid #101828 Inter and the
Alerts colored stat borders go neutral. Semantic up/down cell colors kept.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11811,6 +11811,33 @@
       <c r="E109" t="inlineStr">
         <is>
           <t>Frontend rebuilt + recreated (:3004 healthy). Verified. Ready to commit/push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Portfolio pages: simplify grids + de-colourise (Holdings, Alerts)</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Holdings (.portfolio-table, holdings.css) and Alerts (.alerts-table, alerts.css) had gradient headers (purple / orange-&gt;red), zebra rows, scale hover, and gradient-text stat values. Appended unified overrides at end of each css: thead -&gt; #fafafa subtle gray, header th #475467 12px no-gradient, td border-bottom 1px #e4e7ec + 13px, rows white (no zebra), hover #f9fafb no transform. De-colourised the decorative gradient-text values (.summary-value / .stat-value) to solid #101828 Inter; Alerts colored stat-card bottom borders -&gt; neutral #e4e7ec. Performance is charts (no grid); Watchlist already unified.</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Same approach as the Stocks fix (append override last + !important to beat the gradient rules). Semantic up/down cell colours not touched. User chose to commit without screenshot verification.</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + recreated (:3004 healthy). Committed; not yet visually verified by screenshot (user opted to commit). Ready to push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ui): compact Holdings title, summary cards and table rows
Per request: shrink the "My portfolio" heading to 14px, reduce the
Total value / Total stocks summary card padding + value/icon sizes so the
row is shorter, and tighten table cell padding (1rem -> 6px) so data rows
are less tall.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11838,6 +11838,33 @@
       <c r="E110" t="inlineStr">
         <is>
           <t>Frontend rebuilt + recreated (:3004 healthy). Committed; not yet visually verified by screenshot (user opted to commit). Ready to push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Holdings: compact title, summary cards &amp; table rows</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Per request, reduced sizes on Holdings (holdings.css override): .page-header h1 "My portfolio" 1.25rem-&gt;14px; .summary-card padding 1.25/1.5rem-&gt;10/14px; .summary-item padding 0.5/1rem-&gt;6/12px, no hover lift; .summary-icon 2.5rem-&gt;1.75rem; .summary-value 1.375rem-&gt;15px; .summary-item h3 11px; .portfolio-table thead th padding -&gt;8/12px; tbody td padding 1rem/1.25rem-&gt;6/12px. Result: smaller title, shorter Total value/Total stocks row, shorter data rows.</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Verified by screenshot. Remaining colourful cell pills (Symbol=blue, Shares=green, Price=teal, Total value=amber) are .td-* badges still coloured; not changed this turn (user asked only about sizes). Could flatten them next if wanted, per earlier "data item not colourful" note.</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + recreated (:3004 healthy). Holdings sizes verified. Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): flatten Holdings cell pills to plain text
Remove the coloured pill styling from the Holdings table cells:
.symbol-badge -> plain blue link; .shares-badge / .price-value /
.total-value-badge -> plain #344054 text (drop background, border,
radius, shadow, padding) and hide the small currency/coin icons.
Semantic up/down colors are untouched.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F111"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11865,6 +11865,33 @@
       <c r="E111" t="inlineStr">
         <is>
           <t>Frontend rebuilt + recreated (:3004 healthy). Holdings sizes verified. Ready to commit/push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Holdings: flatten coloured cell pills to plain text</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Flattened the Holdings table cell badges to plain text in holdings.css: .symbol-badge (blue pill)-&gt;plain blue link; .shares-badge (green pill), .price-value (teal pill+border #99f6e4), .total-value-badge (amber pill+border #fcd34d+shadow)-&gt;plain #344054 text. Removed background/border/border-radius/box-shadow/padding and hid the small decorative currency/coin icons (.price-value&gt;svg, .total-value-badge&gt;svg, .currency-icon). Semantic .positive/.negative not touched.</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Verified by screenshot: Symbol blue link, Shares/Price/Total value plain text, no boxes/icons. Remaining minor colour: summary-card top gradient bar + two small icon chips (green/indigo) in the Total value/Total stocks row — left as-is (not table cells).</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + recreated (:3004 healthy). Verified. Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): unify SimulationDashboard transaction table to Holdings style
Last colourful data table: .transaction-table had a purple gradient
uppercase header and buy/sell pill badges. Switch to the shared look —
gray #fafafa header, #475467 12px sentence-case, #e4e7ec row dividers,
13px cells, calm hover — and flatten .badge-buy/.badge-sell to plain
colored text. Price Board (.custom-table) remains untouched.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F112"/>
+  <dimension ref="A1:F113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11892,6 +11892,33 @@
       <c r="E112" t="inlineStr">
         <is>
           <t>Frontend rebuilt + recreated (:3004 healthy). Verified. Ready to commit/push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Project-wide: all data tables match the Holdings style</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Swept all data tables for colourful styling. Only remaining outlier was SimulationDashboard .transaction-table (purple gradient header, uppercase, buy/sell pill badges) in SimulationDashboard.css -&gt; changed to gray #fafafa header, #475467 12px sentence-case, #e4e7ec dividers, 13px cells, calm hover; .badge-buy/.badge-sell flattened to plain colored text (semantic). All other tables already conform: component.css .table and journal.css .trade-table and Watchlist use clean #f9fafb headers; everything else uses the theme-ui unified grid. Price Board (.services .custom-table, table_style.css) left untouched (dark terminal).</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Verified via grep sweep: no other -table thead gradients or strongly-coloured headers remain; only neutral inline cell is RiskDashboard correlation-matrix diagonal (#f3f4f6 gray, intentional). Served CSS confirms transaction-table thead = #fafafa (gradient removed).</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Frontend rebuilt + recreated (:3004 healthy, css main.eb4ee2f7.css). Project data tables unified. Ready to commit/push.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(deploy): auto-detect host IP so remote access works zero-config
The frontend bakes REACT_APP_API_URL at build time, so a localhost-only
value broke access from other machines. Make the compose build arg read
${REACT_APP_API_URL:-http://localhost:18004}, and in deploy-interactive.sh:

- detect_host_ip() / resolve_api_url(): use the host's LAN IP (default-route
  src, fallback hostname -I, then localhost); an explicit REACT_APP_API_URL
  env var overrides.
- ensure_stock_env() writes REACT_APP_API_URL into stockpredict/.env and, when
  it changes, flags a frontend rebuild (the URL is compiled into the bundle).
- Auto-mode summary prints the http://<host-ip>:3004/stock-app links for LAN
  devices and notes localhost still works on the host.

Verified: bash -n, host-IP detection, and `docker compose config` honoring
the build arg.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8960,7 +8960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11948,6 +11948,34 @@
           <t>deploy-interactive.sh updated (repo root). Usage: ./deploy-interactive.sh --auto. Ready to commit/push.</t>
         </is>
       </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Deploy: auto-detect host IP so remote access works zero-config</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Frontend bakes REACT_APP_API_URL at build time so localhost-only broke remote browsers. Made docker-compose.full-stack.yml frontend build arg read the env var with a localhost default. In deploy-interactive.sh added detect_host_ip (default-route src IP, fallback hostname -I, then localhost) and resolve_api_url (explicit REACT_APP_API_URL env wins, else host IP on port 18004). ensure_stock_env now writes REACT_APP_API_URL into stockpredict/.env for both new and existing files and sets FORCE_FRONTEND_REBUILD when it changes so the frontend rebuilds with the new URL. Auto summary prints the host-IP links for LAN devices.</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Verified bash -n, host IP detection gave 10.1.10.42, and docker compose config honors the build arg. Same value serves local and remote. Network change triggers a rebuild via FORCE_FRONTEND_REBUILD. Override with REACT_APP_API_URL env var.</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>deploy-interactive.sh + docker-compose.full-stack.yml updated and committed (fabc2123 + this). Ready to push.</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(roadmap): log Event-Reaction subsystem (Phases 0-3 complete)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G120"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4658,6 +4658,43 @@
       <c r="G120" t="inlineStr">
         <is>
           <t>Spec: docs/SRS_submodule_multiscale_nesting.md; plan: docs/implementation_plan_fpr_multiscale.md — ALL of Part B (B1–B7) complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Event Reaction</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Surprise-based event study</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Price reaction to the surprise of discrete events (align, surprise, market-model AR/CAR, Lee-Mykland jump, cross-sectional exposure)</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>stock_microservices/event-reaction-lib + services/event-reaction-service</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>62 lib + 7 service tests green; SRS_event_reaction.md v1.1; docs/implementation_plan_event_reaction.md</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Observed surprise (consensus/futures/odds; llm deferred). Daily-only (intraday deferred). Frontend report deferred.</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F115"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11975,7 +12012,33 @@
           <t>deploy-interactive.sh + docker-compose.full-stack.yml updated and committed (fabc2123 + this). Ready to push.</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Event-Reaction subsystem — Phases 0-3 (gap map, SRS, plan, full implementation)</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>New backend subsystem measuring price reaction to the SURPRISE of discrete events. Library stock_microservices/event-reaction-lib (package event_reaction, flat stage packages ingest/align/surprise/returns/jumps/cross_section) + stateful service stock_microservices/services/event-reaction-service (MySQL event store, FastAPI, port 8012, Traefik /stock_helper/api/v2/event-reaction). Docs: docs/event_reaction_gap_map.md, SRS_event_reaction.md (v1.1), docs/implementation_plan_event_reaction.md. 11 gated tasks (T0-T11), committed per task. Reuses chart_decomp estimate_volatility/make_surrogate and stock-data-service /history over HTTP. 62 lib + 7 service tests green.</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Surprise is OBSERVED (consensus default; futures/Kuttner, odds; llm deferred) — NOT modelled. Two domain-bug gates proven: no-look-ahead (post-event mutation inert) and same-day clustering (iid t-test size 0.68 vs cluster/portfolio ~0.09). Lee-Mykland is a daily variant with a single-test threshold (event day pre-specified, not scanned). Nested event-reaction-lib/CLAUDE.md holds module rules; root CLAUDE.md untouched.</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Module complete through T11; all mandatory tests pass. Next-up (deferred): frontend event-reaction report component (new sibling to PatternTab); LLM surprise constructor (v2, chatbot); intraday Lee-Mykland; add service to prod/test/ha compose variants.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
refactor(ui): Event Reaction Overview follows the EN/VI switcher
The Overview tab previously rendered English and Vietnamese together on one
page. Rework it to show a single language driven by the app's i18n switcher,
matching the rest of the app.

Move all Overview copy into i18n (event_reaction.overview.*) in en.json +
vi.json — hero, benefits[], steps[], flow[], glossary[] — and rewrite
OverviewTab to read them via t()/returnObjects. Remove the hardcoded
bilingual arrays and the EN/VI badge tags. Analysis tab unchanged.

Tests updated to assert one-language-at-a-time (active-lang hero present,
other-lang hero absent) — 3/3 pass; CI build clean.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8997,7 +8997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F117"/>
+  <dimension ref="A1:F118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12067,6 +12067,38 @@
         </is>
       </c>
       <c r="F117" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Event Reaction — Overview tab now follows the EN/VI language switcher (single language)</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Reworked the Event Reaction Overview tab so it renders one language at a time via the app's i18n switcher instead of showing English and Vietnamese together. Removed the hardcoded bilingual arrays (BENEFITS/STEPS/GLOSSARY) and the LangTag EN/VI badges from src/components/Pages/EventReaction/index.js; OverviewTab now reads event_reaction.overview.* via t() (hero_title, hero_subtitle, benefits_title, benefits[], howto_title, steps[{title,desc}], flow[], glossary_title, glossary[{term,desc}]) using returnObjects for the arrays. Added the full overview block to both en.json and vi.json (identical structure: 5 benefits, 5 steps, 4 flow chips, 4 glossary terms). Analysis tab unchanged.</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Verified: EventReaction.test.js rewritten to assert one-language-at-a-time (EN hero present AND VI hero absent when lang=en, and the reverse when lang=vi) — 3/3 pass; CI=true npm run build compiles clean (host bundle main.17b15835.js). Rebuilt the frontend Docker image + recreated only stock_frontend (--no-deps): healthy, serving fresh bundle main.b97d03a2.js. Container-built hash differs from the host build because the image runs npm run build internally with the baked REACT_APP_API_URL — expected. i18n bundles both locales in the JS; the switcher selects which renders.</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Overview tab live and localized at http://10.1.10.42:3004/stock-app (Event Reaction -&gt; Overview). Ready to commit/push.</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
         <is>
           <t>None</t>
         </is>

</xml_diff>

<commit_message>
fix(news): auto-create stock_news database on startup for Docker deploys
create_all() makes tables but not the database, and mysql/init only seeds a fresh
volume — so deploying against an existing MySQL failed with 'Unknown database'.
NewsRepository.ensure_schema now runs CREATE DATABASE IF NOT EXISTS first (no-op for
sqlite). Verified end-to-end against the running stock_mysql. Note: url.set(database=None)
is a no-op in SQLAlchemy; use database="" to clear it.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -9076,7 +9076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F130"/>
+  <dimension ref="A1:F131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12504,6 +12504,33 @@
       <c r="E130" t="inlineStr">
         <is>
           <t>STREAM B COMPLETE end-to-end (N1-N10): watched-symbol resolve -&gt; vnstock company news -&gt; ai-insights classify (LLM sentiment+category) -&gt; news_events store (dedup) -&gt; news.company event -&gt; portfolio per-user in-app + email -&gt; React bell UI. Remaining: STREAM A — N11 macro feed adapters (RSS/JSON + tagging), N12 macro poller, N13 event-reaction bridge; then N14 close-out (ROADMAP/MEMORY/smoke). Not committed (commit on user request).</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>News ingestion — deploy fix: auto-create the stock_news database on startup</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Verified the news_events table auto-generates on a Docker deploy — found and fixed a real gap. mysql/init only runs on a FRESH volume, and the running stock_mysql (up 24h) had auth_db/portfolio_db/... but NO stock_news; create_all() makes tables not the database, so news-service startup would fail with Unknown database. Fix: NewsRepository.ensure_schema now calls _ensure_database() first — connects to the server (URL with database cleared) and runs CREATE DATABASE IF NOT EXISTS stock_news (utf8mb4), then create_all. No-op for sqlite.</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Bug caught during live verification: url.set(database=None) is a NO-OP in SQLAlchemy (keeps the original db); must use url.set(database="") to clear it. Proven end-to-end: built stock_microservices-news-service, ran a one-off container on stock-network against stock_mysql (ENABLE_COMPANY=0) -&gt; logs "ensured database stock_news exists" + "startup OK"; stock_mysql now shows the stock_news DB and news_events table with all 17 columns + indexes. Probe removed. news-service suite 68/68 (added a sqlite no-op test). NOTE: event-reaction-service has the identical gap (create_all only, no CREATE DATABASE) — its stock_event_reaction DB was also missing from stock_mysql; recommend the same _ensure_database fix there.</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Deploy auto-generation verified/fixed. Continuing to Stream A: N11 macro feed adapters. Follow-up candidate: apply the same DB-auto-create to event-reaction-service.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(news): N14 close-out — mark module Done + roadmap/session log
End-to-end live smoke passed against stock_mysql (boot healthy, ingest+dedup, read-back,
poll routing, persistence). News Ingestion marked Done in Feature Inventory + Roadmap.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -4721,12 +4721,12 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Design phase done: docs/SRS_news_ingestion.md v1.0 (FR-NEWS-*, EC-N*) + docs/implementation_plan_news_ingestion.md (14 tasks N1-N14, Stream B first). Implementation not started. | N1 done (2026-07-02): news-service scaffold — FastAPI app, config (port 8013, stream toggles), exceptions, package skeleton, Dockerfile, requirements; 6 health/config tests green. | N2 done: news_events store — SQLAlchemy NewsEvent (portable MySQL/sqlite, MEDIUMTEXT variant), NewsItem contract with pure sha256 news_id() (guid&gt;url&gt;composite), NewsRepository insert-if-absent upsert (no-op on re-see) + mark_classified/notified/bridged + list_new/query, UTC tz normalization on read/write. 15 tests green. | N3 done: watched-symbol resolver — news-service app/ingest/watch_source.py (httpx union of portfolio+helper, uppercased/deduped/sorted, resilient to a down upstream, user-agnostic); additive endpoints GET /portfolio/watched-symbols (repo get_all_watched_symbols) + GET /helper/watched-tickers, both cross-user DISTINCT, unauthenticated. news-service 21 tests green + 2 upstream endpoint tests. | N4 done: company-news source adapter app/ingest/company_source.py — CompanyNewsSource.fetch(symbol) calls stock-data GET /companies/{symbol}/news, normalizes each vnstock record to NewsItem (tz-aware UTC ts, raw_json verbatim, body prefers full content, url from vnstock source-link). Non-200/non-list/network -&gt; SourceUnavailableError; empty list = normal no-news; bad records skipped. news-service 30 tests green. | N5 done: classifier adapter app/ingest/classifier.py — NewsClassifier.classify(item) POSTs to ai-insights /ai/news-analysis, maps overall_sentiment-&gt;{good,bad,neutral} + sentiment_score clamped[-1,1]; category keyword-derived locally (EN+VI) since ai-insights returns no category; error/timeout-&gt;ClassificationError. news-service 48 tests green. | N6 done: company poller + notifier + scheduler — two-phase tick (ingest: resolve-&gt;fetch-&gt;upsert new; classify+notify: list_new-&gt;classify-&gt;mark-&gt;emit news.company for good/bad only + mark_notified), non-overlapping async PollerScheduler, Notifier over stock-common EventBus (symbol-scoped, no user), wired into main lifespan gated to non-test env. news-service 55 tests green. | Enhancement: ai-insights NewsAnalysisResponse now returns an LLM-assigned category (closed vocab, keyword fallback in ai-insights) and the news-service classifier prefers it over local keywords. ai-insights 206 + news-service 57 green. | N7 done: portfolio-service news.company consumer — NotificationType.NEWS_COMPANY, news_event_handler fans a symbol-scoped event to per-user in-app notifications (repo.get_user_ids_for_symbol join), per-(user,news_id) dedup, optional email to newly-notified users when SMTP configured; registered in lifespan + idempotent MySQL enum ALTER (names, verified vs create_all DDL). portfolio 182 pass (only 2 pre-existing fails). Stream B end-to-end (emit+consume). | N8 done: read API — GET /news (filters stream/symbol/category/sentiment/since/until + paging, list omits raw_json), GET /news/{id} (incl raw_json, 404 if missing), POST /ingest (dedup store, classify/notify on next tick), POST /poll/{stream} (company runs container poller, macro 501, unknown 400). news-service 67 green. | N9 done: docker-compose news-service block (build, env for all upstream URLs + RabbitMQ + stock_news DATABASE_URL + ENABLE_* toggles, expose 8013, healthcheck, 6 Traefik labels PathPrefix /stock_helper/api/v2/news port 8013); mysql/init adds stock_news (+ stock_event_reaction) DB + grants; portfolio news consumer auto-runs in lifespan. docker compose config validates (exit 0). | N10 done: React NotificationBell renders news_company items (Newspaper icon, symbol pill, good/bad sentiment badge, category, "Read more" external link); 16/16 NotificationBell tests, clean CRA build, frontend Docker image rebuilt + stock_frontend recreated (healthy, serving 200). STREAM B COMPLETE (N1-N10). | N11 done (Stream A start): macro feed adapters app/ingest/macro_feeds.py — registry-driven RSS(feedparser)+JSON readers -&gt; (NewsItem, category) TaggedItems, keyword tag_category (monetary/tariff/tax/trade/geopolitical/war/other), tz-aware UTC + raw_json preserved, per-source log-and-continue. feedparser dep added. news-service 81 green. | N12+N13 done (Stream A complete): MacroPoller (fetch_all -&gt; upsert -&gt; mark_classified(category, sentiment=None) so macro rows are tagged and excluded from company classify via list_new(stream); no notify) wired behind ENABLE_MACRO; EventReactionBridge.maybe_bridge posts whitelisted numeric releases (monetary-&gt;rate_decision, tariff, tax) to event-reaction /events with event_id=news_id (idempotent) behind ENABLE_BRIDGE; list_new gained a stream filter; /poll/macro runs the poller. news-service 93 green.</t>
+          <t>Design phase done: docs/SRS_news_ingestion.md v1.0 (FR-NEWS-*, EC-N*) + docs/implementation_plan_news_ingestion.md (14 tasks N1-N14, Stream B first). Implementation not started. | N1 done (2026-07-02): news-service scaffold — FastAPI app, config (port 8013, stream toggles), exceptions, package skeleton, Dockerfile, requirements; 6 health/config tests green. | N2 done: news_events store — SQLAlchemy NewsEvent (portable MySQL/sqlite, MEDIUMTEXT variant), NewsItem contract with pure sha256 news_id() (guid&gt;url&gt;composite), NewsRepository insert-if-absent upsert (no-op on re-see) + mark_classified/notified/bridged + list_new/query, UTC tz normalization on read/write. 15 tests green. | N3 done: watched-symbol resolver — news-service app/ingest/watch_source.py (httpx union of portfolio+helper, uppercased/deduped/sorted, resilient to a down upstream, user-agnostic); additive endpoints GET /portfolio/watched-symbols (repo get_all_watched_symbols) + GET /helper/watched-tickers, both cross-user DISTINCT, unauthenticated. news-service 21 tests green + 2 upstream endpoint tests. | N4 done: company-news source adapter app/ingest/company_source.py — CompanyNewsSource.fetch(symbol) calls stock-data GET /companies/{symbol}/news, normalizes each vnstock record to NewsItem (tz-aware UTC ts, raw_json verbatim, body prefers full content, url from vnstock source-link). Non-200/non-list/network -&gt; SourceUnavailableError; empty list = normal no-news; bad records skipped. news-service 30 tests green. | N5 done: classifier adapter app/ingest/classifier.py — NewsClassifier.classify(item) POSTs to ai-insights /ai/news-analysis, maps overall_sentiment-&gt;{good,bad,neutral} + sentiment_score clamped[-1,1]; category keyword-derived locally (EN+VI) since ai-insights returns no category; error/timeout-&gt;ClassificationError. news-service 48 tests green. | N6 done: company poller + notifier + scheduler — two-phase tick (ingest: resolve-&gt;fetch-&gt;upsert new; classify+notify: list_new-&gt;classify-&gt;mark-&gt;emit news.company for good/bad only + mark_notified), non-overlapping async PollerScheduler, Notifier over stock-common EventBus (symbol-scoped, no user), wired into main lifespan gated to non-test env. news-service 55 tests green. | Enhancement: ai-insights NewsAnalysisResponse now returns an LLM-assigned category (closed vocab, keyword fallback in ai-insights) and the news-service classifier prefers it over local keywords. ai-insights 206 + news-service 57 green. | N7 done: portfolio-service news.company consumer — NotificationType.NEWS_COMPANY, news_event_handler fans a symbol-scoped event to per-user in-app notifications (repo.get_user_ids_for_symbol join), per-(user,news_id) dedup, optional email to newly-notified users when SMTP configured; registered in lifespan + idempotent MySQL enum ALTER (names, verified vs create_all DDL). portfolio 182 pass (only 2 pre-existing fails). Stream B end-to-end (emit+consume). | N8 done: read API — GET /news (filters stream/symbol/category/sentiment/since/until + paging, list omits raw_json), GET /news/{id} (incl raw_json, 404 if missing), POST /ingest (dedup store, classify/notify on next tick), POST /poll/{stream} (company runs container poller, macro 501, unknown 400). news-service 67 green. | N9 done: docker-compose news-service block (build, env for all upstream URLs + RabbitMQ + stock_news DATABASE_URL + ENABLE_* toggles, expose 8013, healthcheck, 6 Traefik labels PathPrefix /stock_helper/api/v2/news port 8013); mysql/init adds stock_news (+ stock_event_reaction) DB + grants; portfolio news consumer auto-runs in lifespan. docker compose config validates (exit 0). | N10 done: React NotificationBell renders news_company items (Newspaper icon, symbol pill, good/bad sentiment badge, category, "Read more" external link); 16/16 NotificationBell tests, clean CRA build, frontend Docker image rebuilt + stock_frontend recreated (healthy, serving 200). STREAM B COMPLETE (N1-N10). | N11 done (Stream A start): macro feed adapters app/ingest/macro_feeds.py — registry-driven RSS(feedparser)+JSON readers -&gt; (NewsItem, category) TaggedItems, keyword tag_category (monetary/tariff/tax/trade/geopolitical/war/other), tz-aware UTC + raw_json preserved, per-source log-and-continue. feedparser dep added. news-service 81 green. | N12+N13 done (Stream A complete): MacroPoller (fetch_all -&gt; upsert -&gt; mark_classified(category, sentiment=None) so macro rows are tagged and excluded from company classify via list_new(stream); no notify) wired behind ENABLE_MACRO; EventReactionBridge.maybe_bridge posts whitelisted numeric releases (monetary-&gt;rate_decision, tariff, tax) to event-reaction /events with event_id=news_id (idempotent) behind ENABLE_BRIDGE; list_new gained a stream filter; /poll/macro runs the poller. news-service 93 green. | N14 close-out: end-to-end live smoke against stock_mysql — service boots healthy, POST /ingest stored + dedup (stored true then false), GET /news reads back tz-aware, /poll company+macro 503 (off) / bogus 400, row persisted then cleaned. MEMORY.md pointer added. DONE.</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -6917,7 +6917,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -9076,7 +9076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F133"/>
+  <dimension ref="A1:F134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12585,6 +12585,33 @@
       <c r="E133" t="inlineStr">
         <is>
           <t>ALL BUILD TASKS DONE (N1-N13). Stream A + Stream B complete. Next-up: N14 close-out — mark Feature Inventory Done, MEMORY.md pointer, end-to-end smoke; then commit Stream A (N11-N13 uncommitted) and push. Follow-up still open: apply the same _ensure_database auto-create to event-reaction-service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>News ingestion — task N14: close-out (smoke + docs) — MODULE DONE</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Marked Feature Inventory "News Ingestion" = Done and Roadmap row Done. Added MEMORY.md pointer + memory/project_news_ingestion.md (ports, DB auto-create gotcha, classification split, event-reaction follow-up). End-to-end live smoke: rebuilt stock_microservices-news-service, ran it against the real stock_mysql on stock-network with a published port — /health/ready 200, POST /ingest returned stored:true then stored:false on re-post (dedup EC-N2), GET /news returned the row with tz-aware ts_utc, /poll/company + /poll/macro = 503 (pollers off), /poll/bogus = 400; verified the row persisted in stock_news.news_events, then deleted the smoke row (DB left clean) and removed the container.</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Whole build N1-N14 complete: news-service 93 tests, plus edits green in portfolio (news_event_handler + repo), ai-insights (+2), decision-helper (+1), frontend NotificationBell (16). Two streams share the news_events corpus; Stream B on by default and deployed to the running frontend, Stream A behind ENABLE_MACRO/ENABLE_BRIDGE. Commits on feat/news-ingestion: 9df7347d (Stream B), 16b1b9ec (DB auto-create fix), 75c35545 (Stream A). N14 roadmap commit pending.</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>NEWS INGESTION MODULE COMPLETE (N1-N14). Open follow-ups: (1) apply the same _ensure_database DB-auto-create fix to event-reaction-service (identical missing-DB gap); (2) enable Stream A by configuring real feed sources + ENABLE_MACRO/ENABLE_BRIDGE; (3) the 3 pre-existing event-reaction design docs remain untracked; (4) 2 pre-existing portfolio test failures (mock/impl drift) still open. Commit ROADMAP.xlsx for N14, then optionally open a PR from feat/news-ingestion.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(event-reaction): auto-create stock_event_reaction database on startup
Same deploy gap as news-service: create_all() makes tables not the database, and
mysql/init only seeds a fresh volume, so deploying against an existing MySQL failed with
'Unknown database'. MySqlEventRepository.ensure_schema now runs CREATE DATABASE IF NOT
EXISTS first (no-op for sqlite). Verified live against the running stock_mysql.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -9076,7 +9076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F134"/>
+  <dimension ref="A1:F135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12612,6 +12612,33 @@
       <c r="E134" t="inlineStr">
         <is>
           <t>NEWS INGESTION MODULE COMPLETE (N1-N14). Open follow-ups: (1) apply the same _ensure_database DB-auto-create fix to event-reaction-service (identical missing-DB gap); (2) enable Stream A by configuring real feed sources + ENABLE_MACRO/ENABLE_BRIDGE; (3) the 3 pre-existing event-reaction design docs remain untracked; (4) 2 pre-existing portfolio test failures (mock/impl drift) still open. Commit ROADMAP.xlsx for N14, then optionally open a PR from feat/news-ingestion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Event-Reaction — deploy fix: auto-create stock_event_reaction database on startup</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Applied the same DB-auto-create fix to event-reaction-service (identical gap to news-service). MySqlEventRepository.ensure_schema now calls _ensure_database() first — connects to the server (URL with database="") and runs CREATE DATABASE IF NOT EXISTS stock_event_reaction (utf8mb4) before create_all; no-op for sqlite. Added a sqlite no-op unit test.</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Verified live: built stock_microservices-event-reaction-service, ran a probe against the real stock_mysql (which had NO stock_event_reaction DB) -&gt; logs "ensured database stock_event_reaction exists" + "event store + price source wired OK"; stock_mysql now shows the stock_event_reaction DB and event_reaction_events table. Probe removed. event-reaction-service tests 8/8 (added the sqlite no-op test).</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Event-reaction DB-auto-create follow-up DONE. News module complete (N1-N14). Remaining open items: enable Stream A feeds; 3 untracked event-reaction design docs; 2 pre-existing portfolio test failures. Commit this fix; optionally PR feat/news-ingestion.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
deploy(news): wire news-service into the full-stack + rebuild portfolio consumer
Adds the news-service block to docker-compose.full-stack.yml (port 8013, Traefik
/stock_helper/api/v2/news, root DB URL for auto-create, ENABLE_COMPANY=1). Deploy also
rebuilds portfolio-service (news.company consumer + /watched-symbols) and
decision-helper-service (/watched-tickers). Verified live: news-service + portfolio
healthy, consumer subscribed, DB auto-created, upstream legs reachable.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -9076,7 +9076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:F136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12639,6 +12639,33 @@
       <c r="E135" t="inlineStr">
         <is>
           <t>Event-reaction DB-auto-create follow-up DONE. News module complete (N1-N14). Remaining open items: enable Stream A feeds; 3 untracked event-reaction design docs; 2 pre-existing portfolio test failures. Commit this fix; optionally PR feat/news-ingestion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>News ingestion — DEPLOYED LIVE into the running full-stack</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Added news-service to docker-compose.full-stack.yml (build from stock_microservices context, container stock_news_service, DATABASE_URL as root-&gt;mysql/stock_news since auto-create needs CREATE DATABASE which stockuser lacks, service-name upstream URLs, RabbitMQ, ENABLE_COMPANY=1 others off, Traefik stock-news port 8013). Rebuilt+recreated portfolio-service (loads the news.company consumer + /watched-symbols endpoint + notifications.type enum ALTER) and decision-helper-service (/watched-tickers), and brought up news-service.</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Verified live end-to-end plumbing: news-service healthy — logs "ensured database stock_news exists" + "scheduler company started (900s)" + startup OK; portfolio healthy — "News consumer subscribed to news.company" on its own durable queue. Gateway routes 200: /portfolio/watched-symbols, /helper/watched-tickers, /news/poll/company. A manual /news/poll/company reached both watched-symbol endpoints (200) and returned fetched:0 because NO user currently holds/watches any ticker (correct). Source+classifier legs confirmed: stock-data /companies/FPT/news returns real vnstock articles; ai-insights /news-analysis returns 200. So the whole chain works; notifications will flow once a user adds a ticker (e.g. FPT/ACB) to portfolio/watchlist — poller picks it up each 15min (or via POST /news/poll/company).</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LIVE. To see a notification: add FPT/ACB to a portfolio holding or watchlist in the app, then wait a poll cycle or trigger POST /stock_helper/api/v2/news/poll/company. Optional: controlled demo (inject a holding+news, poll, show the bell notification, clean up). event-reaction-service still not deployed (bridge off, so not required). Commit docker-compose.full-stack.yml.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(news): fall back to ingestion time when company news lacks a publishDate
vnstock company-news records can carry publishDate=null, which made CompanyNewsSource
skip every item (fetched 0 in a live poll). Since news_id dedup keys on guid/url (not
date), stamp such items at ingestion time instead of dropping real news. Title is still
required. Verified live: a poll then fetched 50 real FPT articles.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -9076,7 +9076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F136"/>
+  <dimension ref="A1:F137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12666,6 +12666,33 @@
       <c r="E136" t="inlineStr">
         <is>
           <t>LIVE. To see a notification: add FPT/ACB to a portfolio holding or watchlist in the app, then wait a poll cycle or trigger POST /stock_helper/api/v2/news/poll/company. Optional: controlled demo (inject a holding+news, poll, show the bell notification, clean up). event-reaction-service still not deployed (bridge off, so not required). Commit docker-compose.full-stack.yml.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>News ingestion — controlled live end-to-end demo + null-date fix</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Ran a controlled end-to-end demo on the running stack against the default portfolio (user_id=1, portfolio_id=1). Found ai-insights runs template-only (no LLM key) so it returns neutral even for strongly-positive text -&gt; real classifier path never yields good/bad here. Also found+fixed a real bug: vnstock company news returns publishDate=null, so CompanyNewsSource skipped ALL items (fetched 0). Fix: title still required, but a missing/unparseable date now falls back to ingestion time (dedup keys on guid/url not date, so safe) instead of dropping real news. Updated the test accordingly. Rebuilt+redeployed news-service.</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>After the fix, a live POST /news/poll/company fetched 50 real FPT articles, stored+deduped+classified (neutral, template LLM; keyword categories new_tech/other), notified 0 (correct — neutral). Then published the exact news.company (sentiment=good) event news-service emits under a real LLM via the news container EventBus -&gt; portfolio consumer logged "fanned to 1 user(s) (1 new)" and created notification id for user 1 (type NEWS_COMPANY, title "Good news for FPT", unread). Verified via DB. Teardown restored exact baseline: 0 notifications, 0 holdings, 0 news_events rows. news-service suite still 93/93.</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>DEMO SUCCESSFUL — full chain proven live (ingest+classify+store real FPT news; notify fan-out to the bell). To get good/bad classification (and thus real auto-notifications), configure an LLM key for ai-insights (currently template-only -&gt; everything neutral). To use for real: add FPT/ACB to a portfolio/watchlist in the app. Commit the null-date fallback fix.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(news): enable Stream A macro feeds + event-reaction bridge
Flip news-service ENABLE_MACRO/ENABLE_BRIDGE 0->1 in the full-stack compose
(overridable via NEWS_ENABLE_MACRO/NEWS_ENABLE_BRIDGE), add MACRO_POLL_INTERVAL
and a FEED_REGISTRY_PATH passthrough.

Macro poller now fetches Fed-press items into the news corpus (GET
/news/news?stream=macro). Bridge is wired but posts 0 events with the default
RSS press-release sources (no numeric actual/consensus); auto-populating the
Measure event list requires a JSON economic-calendar feed via FEED_REGISTRY_PATH.

Verified: forced poll fetched=20, tagged=20, bridged=0; corpus returns monetary
items.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -9076,7 +9076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F140"/>
+  <dimension ref="A1:F141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12789,6 +12789,38 @@
       <c r="F140" t="inlineStr">
         <is>
           <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Enable news Stream A (macro feeds) + event-reaction bridge</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Flipped news-service ENABLE_MACRO/ENABLE_BRIDGE 0-&gt;1 in docker-compose.full-stack.yml (now ${NEWS_ENABLE_MACRO:-1}/${NEWS_ENABLE_BRIDGE:-1}); added MACRO_POLL_INTERVAL_SECONDS and FEED_REGISTRY_PATH passthrough. Recreated news-service (config-only, no rebuild). Macro scheduler starts (interval 1800s); a forced POST /news/poll/macro fetched 20 Fed-press items, tagged monetary, stored in corpus. Visible at GET /stock_helper/api/v2/news/news?stream=macro (note doubled news/news path).</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Default macro sources are Fed/Treasury RSS press releases = free text, no numeric actual/consensus, so bridge posts 0 events (event-reaction store still empty) — expected. Treasury feed URL is dead (404). To auto-populate the Measure event list, need a JSON economic-calendar source (actual+consensus/forecast) wired via NEWS_FEED_REGISTRY_PATH; bridge whitelist = monetary-&gt;rate_decision, tariff, tax (KIND_MAP).</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>DONE + verified: macro poll fetched=20 tagged=20 bridged=0; corpus query returns monetary items. Config change is UNCOMMITTED. Next: supply a numeric JSON calendar feed to get bridged/measurable events, and replace the dead treasury_press URL.</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>No frontend page surfaces macro news yet (API only). Bridged events depend on a numeric feed not yet configured.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): log the portfolio summary fix and the price-refresh gap
Sessions Log: 2026-09-09 row covering the holdings summary 0/0 fix — root
cause (field-name mismatch, not a hardcoded zero), the NULL current_value
follow-on, and the live verification against portfolio 1.

Backlog: new #43 — nothing calls POST /portfolios/{id}/refresh-prices, so
holdings keep current_price/current_value NULL and Total Value stays at cost
basis with P&L pinned at 0. Also flags that the quotes URL builds as
STOCK_DATA_SERVICE_URL/{API_PREFIX}/api/v2/stocks/quotes, which looks doubled
and is untested.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EYtXih8Q84RXzXqVwy786z
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -6977,7 +6977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8493,6 +8493,41 @@
       <c r="G43" t="inlineStr">
         <is>
           <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>services/portfolio-service/app/services/portfolio_service.py:204 refresh_prices</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Nothing ever calls POST /portfolios/{id}/refresh-prices, so holdings keep current_price/current_value NULL and the summary falls back to cost basis (P/L always 0). Wire a refresh on load (or a scheduled/event-driven update off stock.price_updated), and check the quotes URL — it builds as STOCK_DATA_SERVICE_URL/{API_PREFIX}/api/v2/stocks/quotes, which looks doubled and is untested.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Portfolio Total Value and P/L are cost basis, not market value — found while fixing the 0/0 summary cards on 2026-09-09.</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -9076,7 +9111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:F142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12821,6 +12856,38 @@
       <c r="F141" t="inlineStr">
         <is>
           <t>No frontend page surfaces macro news yet (API only). Bridged events depend on a numeric feed not yet configured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Fix Portfolio holdings summary showing 0 / 0</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>api.js getPortfolioSummary now maps the backend PortfolioSummary shape (total_holdings/current_value/total_invested) onto the total_stocks/total_value names Holdings.js reads. portfolio_repository.get_portfolio_stats now values a holding at total_cost when current_value is NULL instead of 0. Rebuilt+restarted portfolio-service and frontend images.</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Root cause was a field-name mismatch, not a hardcoded zero: the summary card read summaryResult.data.total_stocks/total_value, which the API never returns, so the || 0 fallbacks always won. Second, latent bug: current_value is a stored column only written by POST /refresh-prices, so it is NULL for every freshly added holding — that also made total_profit_loss read as -100%.</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>DONE + verified against live data (user 1, portfolio 1, one POW holding 150 @ 12850): summary endpoint now returns total_holdings=1, current_value=1927500, profit_loss=0. Cards should show 1 and 1.927.500 VND, matching the table row. Changes are UNCOMMITTED.</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Prices are still never refreshed automatically — nothing calls POST /portfolios/{id}/refresh-prices, so Total Value stays at cost basis until it is wired up (and that URL builds as STOCK_DATA_SERVICE_URL/{API_PREFIX}/api/v2/stocks/quotes, which looks doubled and is untested).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): close Backlog #43 and log the price-refresh fix
Backlog #43 -> Done, with the root cause (dead /stocks/quotes endpoint,
not a malformed URL) and the thousands-quote unit contract recorded.
Sessions Log row for 2026-09-09 noting the remaining gap: refresh runs on
summary reads only, so a scheduled or stock.price.updated-driven refresh
is still the fuller fix.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EYtXih8Q84RXzXqVwy786z
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -8517,12 +8517,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Portfolio Total Value and P/L are cost basis, not market value — found while fixing the 0/0 summary cards on 2026-09-09.</t>
+          <t>Portfolio Total Value and P/L are cost basis, not market value — found while fixing the 0/0 summary cards on 2026-09-09. | 2026-09-09 FIXED: refresh_prices was POSTing to stock-data-service /stocks/quotes, an endpoint that does not exist, so every call 404d, was swallowed by a bare except, and returned 0. Rewritten to read the shared stock_prices tables via the existing repo.get_latest_prices_for_symbols (no HTTP), scaling the thousands-quote close by 1000 to actual VND — the same conversion get_alerts already applies. get_portfolio_summary now calls it best-effort before computing stats, so a summary read marks the portfolio to market; failures degrade to cost basis. NOTE: the URL was NOT doubled — /stock_helper/api/v2/... matches the project convention; the endpoint simply was not there. 5 new unit tests + 2 summary tests; 58 pass in test_portfolio_service_unit.py, 185/186 service-wide (1 pre-existing unrelated failure in test_get_default_portfolio_returns_row_or_none).</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -9111,7 +9111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F142"/>
+  <dimension ref="A1:F143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12888,6 +12888,38 @@
       <c r="F142" t="inlineStr">
         <is>
           <t>Prices are still never refreshed automatically — nothing calls POST /portfolios/{id}/refresh-prices, so Total Value stays at cost basis until it is wired up (and that URL builds as STOCK_DATA_SERVICE_URL/{API_PREFIX}/api/v2/stocks/quotes, which looks doubled and is untested).</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Backlog #43 — make portfolio prices actually refresh</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>portfolio_service.refresh_prices rewritten to source prices from the shared companies+stock_prices tables through the existing repo.get_latest_prices_for_symbols instead of an HTTP POST to a non-existent /stocks/quotes endpoint; scales thousands-quote to actual VND (x1000). get_portfolio_summary now refreshes best-effort before reading stats, wrapped so a price outage degrades to cost basis. Replaced the 3 httpx-mocked refresh tests with 5 DB-path tests (incl. the x1000 unit contract and the no-quotes case) plus 2 summary tests. Rebuilt + restarted portfolio-service.</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>The dead endpoint was the real defect, not the URL shape — /stock_helper/api/v2/stocks/quotes matches convention, stock-data-service just never exposed it (its price surfaces are /priceboards and /stocks/{symbol}/history). Prices were already reachable without HTTP: get_latest_prices_for_symbols joins the stock-data tables in the same MySQL. Unit contract matters — stock_prices.close is a thousands-quote (12.75 = 12,750 VND) while holdings store actual VND; missing the x1000 would understate value 1000x. Writing 0 for an unpriced symbol would report a total loss, so no-quote symbols are left NULL for the cost-basis fallback.</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>DONE + verified live: POW 150 @ 12,850 cost, latest close 12.75 -&gt; current_value 1,912,500, P/L -15,000 (-0.78%), persisted to portfolio_holdings. Summary endpoint returns market value instead of cost basis. UNCOMMITTED.</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Refresh runs on summary reads only, so the holdings table lags one load behind for current_price (the UI computes its row totals from avgPrice, so not user-visible today). A scheduled or stock.price.updated-driven refresh would be the fuller fix — alert_event_handler already consumes that event and could carry it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): log the technical-indicator N/A fix as Backlog #45
Feature Inventory rows 34 and 98 updated with the indicators now served
and the note that the N/A values were a backend field-shape gap, not a
frontend defect. Sessions Log records the root cause, the two latent
bugs found alongside (period-as-calendar-days, inverted S/R) and the
remaining cosmetic issue: formatCurrency prefixes "$" on thousands-quote
VND figures.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VaZaJyQPViTQHiBBDThjFv
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -1892,10 +1892,14 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>RSI/MACD/SMA/support-resistance</t>
-        </is>
-      </c>
-      <c r="G34" s="14" t="inlineStr"/>
+          <t>RSI/MACD/Stochastic/BB/ATR/OBV + SMA20/50/200, clustered S/R, Fibonacci, per-indicator signals (2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="inlineStr">
+        <is>
+          <t>Grouped payload (momentum/volatility/volume/support_resistance/fibonacci_levels) added so the UI Indicators tab renders values, not N/A</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
@@ -3956,12 +3960,12 @@
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>Line 727: TODO Apply indicators to chart</t>
+          <t>Indicators tab reads the grouped fields the API now returns</t>
         </is>
       </c>
       <c r="G98" s="14" t="inlineStr">
         <is>
-          <t>Indicators not yet rendered on chart</t>
+          <t>2026-09-10: N/A values traced to missing backend fields, fixed backend-side; no frontend change needed</t>
         </is>
       </c>
     </row>
@@ -7014,7 +7018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8598,6 +8602,41 @@
         </is>
       </c>
       <c r="G45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>services/analysis-service/app/services/analysis_service.py:341</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Technical Analysis Indicators tab showed N/A for RSI/MACD/Stoch/BB/ATR/OBV/volume, empty S-R and Fibonacci tables, and an empty signal grid</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Response only carried a flat indicators list; the UI reads momentum_indicators / volatility_indicators / volume_indicators / support_resistance / fibonacci_levels / trading_analysis.signals. Also: only `period` calendar days were fetched, so SMA_200 was always null, and _find_support_resistance returned supports above resistances.</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
         <is>
           <t>M</t>
         </is>
@@ -9183,7 +9222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F144"/>
+  <dimension ref="A1:F145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13024,6 +13063,38 @@
       <c r="F144" t="inlineStr">
         <is>
           <t>Claude-side Gmail connector authenticated but then reported "needs to be connected in claude.ai" on every call, so no real emails were read — the SRS is designed against two pasted samples (7 Sep session). Golden set must be built from real .eml files before E2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Fix N/A values in Analysis -&gt; Technical Analysis, Indicators tab</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>analysis-service: added MomentumIndicators / VolatilityIndicators / VolumeIndicators / SupportResistance / TradingSignal schemas plus fibonacci_levels and trading_analysis.signals to TechnicalAnalysisResponse. New helpers _calculate_stochastic, _calculate_obv, _calculate_fibonacci_levels, _safe_float. get_technical_analysis now fetches a 200-bar warm-up run ahead of the display window (CALENDAR_DAYS_PER_BAR=1.6) and trims to `period` bars for the chart. _find_support_resistance rewritten to delegate to the existing clustered _find_sr_levels (F-003) and split levels around current price, nearest-first. 14 new/updated unit tests; 137 pass. Rebuilt + restarted analysis-service.</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>The values were never missing from the database — POW/VNM hold 665 clean OHLCV bars back to 2024-01-02. The UI read grouped field names (momentum_indicators.RSI, volatility_indicators.BB_Upper, volume_indicators.OBV, support_resistance.*, fibonacci_levels, trading_analysis.signals) that the response never contained, so every ?. lookup fell to N/A. Two latent bugs surfaced alongside: `period` was passed to the history API as CALENDAR days, so a 100-bar request returned only 68 trading bars and SMA_200 was permanently null; and the old _find_support_resistance took the 3 highest troughs as supports and the 3 lowest peaks as resistances regardless of price, so it returned supports ABOVE resistances (POW: supports 13.9/14.1/14.6 vs resistances 13.6/13.7/13.85 at a price of 12.75) — which also fed key_levels.support_1 on /summary.</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>DONE + verified live on POW: momentum/volatility/volume groups all populated, SMA_200=13.49, support 12.55 below price and resistances 12.90/13.30/13.75 above, 7 Fibonacci levels, 9 signal rows, chart now 100 bars instead of 68. /summary and /compare re-smoke-tested. No frontend change was needed, so no React rebuild. UNCOMMITTED.</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>TechnicalAnalysis.js formatCurrency prefixes "$" on what are thousands-quote VND figures (12.75 = 12,750 VND) — cosmetic, left alone, and the same unit trap as Backlog #43.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): log Backlog #50 — stale pooled MySQL connections behind the recurring N/A
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011FQyonchEQBTGj7DdpZmLR
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -7018,7 +7018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8777,6 +8777,41 @@
         </is>
       </c>
       <c r="G50" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>stock-common/stock_common/database/connection.py install_stale_connection_guard(); services/*/app/api/dependencies.py</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Stale pooled MySQL connections after an idle gap (wait_timeout=8h) -&gt; first requests return HTTP 500 -&gt; Indicators tab all N/A, Dashboard empty. Recurred every morning; 7 services affected. pool_pre_ping cannot catch asyncmy/uvloop bare RuntimeError; fixed with a pool checkout listener raising DisconnectionError + pool_recycle=1800, and analysis save_analysis made best-effort.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>This is why #45 looked "fixed last week, broken today": the indicator math was right, the DB socket underneath was dead. Verified by KILLing all app connections in MySQL and hitting every dashboard/indicator endpoint first-try.</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
         <is>
           <t>S</t>
         </is>
@@ -9362,7 +9397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F146"/>
+  <dimension ref="A1:F147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13267,6 +13302,38 @@
       <c r="F146" t="inlineStr">
         <is>
           <t>Local only — production deploy is the user's call.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Technical Analysis Indicators N/A recurrence + Dashboard empty on open (Backlog #50)</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>stock-common: install_stale_connection_guard(engine) + ping_or_discard() in database/connection.py, exported; DatabaseManager uses it, pool_recycle 3600-&gt;1800. All 7 services (analysis, stock-data, portfolio, auth, journal, prediction, decision-helper) dependencies.py: pool_recycle=1800 + guard; removed the wrong "pool_pre_ping breaks asyncmy" comment. analysis-service: save_analysis wrapped best-effort (warn + rollback, never 500). Tests: stock-common/tests/test_stale_connection_guard.py (4), test_technical_analysis_survives_cache_write_failure. Rebuilt + restarted the 7 containers. Commit 452f8ca6.</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Indicator math and DB data were fine; #45 was genuinely fixed. The N/A wall was HTTP 500 from a dead pooled MySQL socket: MySQL wait_timeout=8h kills idle connections overnight, asyncmy under uvloop then raises a bare RuntimeError("TCPTransport closed") that SQLAlchemy does NOT classify as a disconnect, so pool_pre_ping=True runs the ping, gets the RuntimeError, and propagates it instead of reconnecting. The fix has to be a pool "checkout" listener that converts ANY ping failure into exc.DisconnectionError (pool then retries with a fresh connection). Reproduce any time with: KILL every non-root id in information_schema.processlist, then curl an endpoint once.</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>DONE + verified locally via :18004 — after a server-side KILL of all app connections, first-try 200 on analysis/technical/POW, stocks/history, portfolios/default, /holdings, /watchlist, ai long/short-term, auth/login; "Discarding stale DB connection" logged once per service, 0 ASGI exceptions. Two pre-existing unit failures untouched: #47 (stock-data financials fixtures) and portfolio test_get_default_portfolio_returns_row_or_none. Uncommitted user edit in TechnicalAnalysis.js (formatCurrency "$" -&gt; "VND") left as-is; needs a frontend image rebuild if wanted. Production machine NOT touched — needs the same rebuild of the 7 services there.</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Production (stock.tuan1970.com) runs on another machine; this fix only lands there after a git pull + rebuild.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): log Backlog #51 (AI Analysis fix) and #52 (repeated N-day prediction)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011FQyonchEQBTGj7DdpZmLR
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -7018,7 +7018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8814,6 +8814,76 @@
       <c r="G51" t="inlineStr">
         <is>
           <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Backend+Frontend</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>services/ai-insights-service/app/services/insights_service.py (_indicator_signal, _effective_date_range, _get_predictions); services/prediction-service/app/services/prediction_service.py predict(); AIInsights.js</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>AI Analysis: indicator dropdowns ignored (score read only RSI+MACD); prediction card frozen because /predictions/predict 404s and prediction-service crashed on sma_50 with 60 calendar days; per user, too-short ranges now auto-widen (end=today-1, start=end-required, MACD≈200d) and the UI shows the effective dates.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>User reported "Analyze changes nothing". Dates already worked; indicators and predictions did not.</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>services/prediction-service/app/services/prediction_service.py predict() loop</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Multi-day forecast feeds the SAME last_row to the model for each of the N days, so day 1..N predictions are identical (only the date differs). Either roll features forward with the predicted close or train per-horizon models.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>The 5-day prediction table shows one number five times.</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -9397,7 +9467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F147"/>
+  <dimension ref="A1:F148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13334,6 +13404,38 @@
       <c r="F147" t="inlineStr">
         <is>
           <t>Production (stock.tuan1970.com) runs on another machine; this fix only lands there after a git pull + rebuild.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>AI Analysis "Analyze does nothing" (Backlog #51)</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>ai-insights: _indicator_signal() scores the selected indicator per category; _analyze_sentiment_from_indicators(df, indicators); _get_predictions fixed to /predict/predict/{symbol} + df-driven _simple_trend_prediction fallback; _effective_date_range/_required_calendar_days auto-widen; schema+route expose effective_start_date/effective_end_date/date_range_adjusted/date_range_note. prediction-service: _inference_lookback_days(), _prepare_features(with_target=False), missing-feature guard, current price from /stocks/{symbol}. React AIInsights.js copies effective dates into the inputs + amber notice; en/vi i18n keys range_adjusted/no_data. Rebuilt ai-insights, prediction, frontend. Commit after 8eace9cb.</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Dates were always honoured (risk score changed with range) — the visible "nothing changes" came from the two sections that never varied: sentiment (RSI+MACD only) and the prediction card (404 -&gt; constant fallback). Calendar-vs-trading-day confusion strikes again (LOOKBACK_PERIOD=60 calendar days cannot fill sma_50). REQUIRED_BARS table x1.6 +14 gives MACD 206 calendar days, matching the user's "200 days" example.</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>DONE + verified live on VIC via :18004. Follow-up logged as Backlog #52: prediction loop repeats one value for all N days. Production machine still needs pull + rebuild of analysis/stock-data/portfolio/auth/journal/prediction/decision-helper/ai-insights + frontend.</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Production is on another machine.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): log AI Analysis on-change widening + default range
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011FQyonchEQBTGj7DdpZmLR
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -9467,7 +9467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F148"/>
+  <dimension ref="A1:F149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13436,6 +13436,38 @@
       <c r="F148" t="inlineStr">
         <is>
           <t>Production is on another machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>AI Analysis follow-ups: on-change date widening + sane default range</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>ai-insights /insights/indicators/available now carries required_calendar_days per indicator (MACD 206, EMA 142, SMA 126, RSI 78, rest 62). AIInsights.js: ensureRangeForSelection() runs on every dropdown change and once when the table loads; default dateRange = last 206 days ending yesterday (was hardcoded 2024). Verified with Playwright (scratchpad pw_ai.py / pw_analyze.py) logged in as the user. Commits 6616c3e2 + this one.</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>User "does not see the dates change" because the old default (2024-01-01..2024-12-31) was already longer than any requirement, so the widen-only rule had nothing to do — and it was analysing 2024 data. nginx cache headers are correct (index.html no-store, hashed bundles immutable), so a plain reload picks up new builds. Playwright (python, chromium) is installed on this host and works against :3004 — the login form username input is NOT type=email.</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>DONE + verified in-browser. Unpushed commits after the user's push: 6616c3e2 and the default-range fix. Production still needs pull + rebuild.</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Production on another machine.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(roadmap): correct the F3 note — deploy-interactive.sh does exist
It sits at the PARENT repo root (/home/tuanph/TuanPH/all_projects/), not inside
stockpredict/. F3's search ran `find . -maxdepth 3` from inside stockpredict/
and never looked up a level, so commit f8deb6bc's message states the opposite.
That history is pushed and is left alone rather than rewritten; the Sessions
Log now carries the correction.

No operational consequence: ./deploy.sh --build is a valid entrypoint and is
what F3 ran, with all 21 services healthy. But deploy-interactive.sh --auto is
the preferred one-command path, because it also generates the gitignored .env
with a fresh JWT secret, bakes the detected LAN IP into REACT_APP_API_URL so
the app reaches other machines, and force-rebuilds the frontend image.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -10634,7 +10634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F167"/>
+  <dimension ref="A1:F168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15195,7 +15195,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Rebuilt every backend and frontend image with ./deploy.sh --build (no deploy-interactive.sh in this repo - that memory was from the other machine; the entrypoint here is deploy.sh). All 21 compose services up and healthy. NEW stock_microservices/scripts/verify-em1-volume.sh - a repeatable deploy check that asserts the endpoint answers through the gateway, that volume is actually read and moves confidence on real bars, and that the SERVED frontend bundle contains the new strings. ROADMAP: Feature Inventory 134 -&gt; Done for backend+frontend, NEW Backlog #72.</t>
+          <t>Rebuilt every backend and frontend image with ./deploy.sh --build (CORRECTION: deploy-interactive.sh DOES exist, at the PARENT repo root /home/tuanph/TuanPH/all_projects/deploy-interactive.sh - NOT inside stockpredict/. I searched only within stockpredict/ and wrongly concluded it was missing. ./deploy.sh --build works and is what was used here, but deploy-interactive.sh --auto is the preferred one-command path: it also generates stockpredict/.env, bakes the LAN IP into REACT_APP_API_URL, and force-rebuilds the frontend image). All 21 compose services up and healthy. NEW stock_microservices/scripts/verify-em1-volume.sh - a repeatable deploy check that asserts the endpoint answers through the gateway, that volume is actually read and moves confidence on real bars, and that the SERVED frontend bundle contains the new strings. ROADMAP: Feature Inventory 134 -&gt; Done for backend+frontend, NEW Backlog #72.</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -15209,6 +15209,38 @@
         </is>
       </c>
       <c r="F167" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Correction to the F3 session note (no code change)</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Corrected the claim that deploy-interactive.sh is absent from this repo.</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>IT EXISTS, one level ABOVE stockpredict: /home/tuanph/TuanPH/all_projects/deploy-interactive.sh. The F3 search used `find . -maxdepth 3` from inside stockpredict/, so it never looked at the parent, and commit f8deb6bc's message repeats the wrong claim - history is pushed and left alone rather than rewritten, so this row is the correction of record. WHICH TO USE: ./deploy.sh --build (inside stockpredict/) is valid and is what F3 actually ran - 21 services came up healthy. But ../deploy-interactive.sh --auto is the preferred entrypoint because it additionally generates the gitignored stockpredict/.env with a fresh JWT secret, bakes the detected LAN IP into REACT_APP_API_URL so the app works from other machines, and force-rebuilds the frontend image. For ONE service, from the PARENT root: docker compose -f stockpredict/docker-compose.full-stack.yml build &lt;svc&gt; &amp;&amp; ... up -d --no-deps &lt;svc&gt; (--no-deps matters, or Compose recreates MySQL/Redis/RabbitMQ too).</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>No action outstanding. EM-1 backend + frontend remain complete and pushed (HEAD 19ca1eb1); S1 and S2 are next. UI placement confirmed with the user: no new menu entry - F1 lives in the existing Chart Patterns panel on Decision Console, F2 is a new card on the existing AI Insights screen. User reviewed and approved keeping it there.</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
         <is>
           <t>None.</t>
         </is>

</xml_diff>

<commit_message>
docs(em-7): T0 — roadmap rows and requirement wiring
Feature Inventory row for EM-7, carrying the two things a future reader needs
and would not find in the code: why the anchor is a broken S/R level rather
than a pattern neckline (ai-insights patterns are unmeasurable in the harness,
and chart-decomp-lib would have the backtest measuring a different detector
than production runs), and what that cost — the trendline half, which E&M rate
highest, needs EM-5.

Idempotence guard added so re-running T0 raises rather than duplicating the
row.

No code.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G137"/>
+  <dimension ref="A1:G138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5291,6 +5291,43 @@
       <c r="G137" s="4" t="inlineStr">
         <is>
           <t>The book itself distrusts measured targets (Ch 32 prefers progressive stops; Bassetti: "decisions should always be made in the here and now, not in the I measured it then"), so the likely deliverable is RETIRING or demoting the MEASURED_MOVE path rather than extending it. Criterion (b) is expectancy not completion, because completion rate is gameable by shrinking the target. Clustering is BY SYMBOL here - a per-symbol treatment, unlike EM-6 market-wide gate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="110" customHeight="1">
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>decision-helper-service</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>EM-7 (FR-EM-T*) Throwback / pullback entry at a broken boundary - E&amp;M Ch 6, Ch 13, Ch 14, tactics in Ch 33</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>services/decision-helper-service/app/services/backtest/market_features.py (break-aware levels, T1) + a new detector in app/services/signal/trend/ (T3); studies in tests/</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F138" s="4" t="inlineStr">
+        <is>
+          <t>Design docs/SRS_edwards_magee_throwback.md v1.0; plan docs/implementation_plan_em7_throwback.md (T0-T5, two gates). ANCHORED ON A BROKEN S/R LEVEL WITH ROLE REVERSAL, not on a pattern neckline: option A (ai-insights patterns) is unmeasurable in the harness, which makes no per-bar HTTP calls, and that is exactly the dead-path trap EM-8 M3 found in MEASURED_MOVE; option B (chart-decomp-lib in-process) would have production and the backtest running DIFFERENT detectors for the same pattern. Ch 13 says "pattern resistance - the mechanism explains the patterns", so the level IS the cause and anchoring there is faithful rather than second-best. Pairs with shipped code: SR_BREAKOUT fires on the break, EM-7 on the return to the same level. No DB change.</t>
+        </is>
+      </c>
+      <c r="G138" s="4" t="inlineStr">
+        <is>
+          <t>TRENDLINE throwbacks are OUT OF SCOPE and that is the half E&amp;M rate highest ("more frequently ... more exactly ... no one knows why") - it needs EM-5 (#65), not built, so EM-7 tests the WEAKER claim and must be reported that way. GATE 1 (T2) needs only T1 and can close #67 in two sessions: the return rate must beat a BAND- AND WINDOW-matched null AND the overshoot must be smaller, since E&amp;M make two claims not one. GATE 2 (T4) is net P&amp;L per breakout OPPORTUNITY with declines counted as zero - average entry price is explicitly not evidence. Standing risk: this is another elaboration on EM-2 levels, and every previous one failed.</t>
         </is>
       </c>
     </row>
@@ -10019,7 +10056,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>midtrend.py has PCT_RETRACEMENT off the swing and LONG_MA_REACTION but nothing anchored to a broken pattern boundary, so a missed breakout stays missed. failed_signal.py covers the opposite case. Benchmark: entry quality vs taking the breakout itself.  || PHASE 1 DESIGN DONE 2026-10-22, docs/SRS_edwards_magee_throwback.md v1.0 (FR-EM-T1..T8, EC-T1..T6, H-T1..H-T8). NOTHING BUILT. FEASIBILITY WAS DECIDED FIRST, BECAUSE EM-8 M3 JUST SHOWED WHY: MEASURED_MOVE was dead code reading a key no detector ever put in signal evidence, so the mechanism could not be measured at all. EM-7 wants a BROKEN PATTERN BOUNDARY at signal time, which is the same class of dependency. Three options weighed: (A) ai-insights patterns_data, already fetched at orchestrator.py:119 - works live but the harness makes NO per-bar HTTP calls by design, so it is UNMEASURABLE and cannot clear C4 - REJECTED as the MEASURED_MOVE trap exactly; (B) add chart-decomp-lib to decision-helper (it has head_shoulders.py, double.py, triangle.py; chart-decomp-service and event-reaction-service already depend on it) - measurable, but production would run ai-insights detector while the backtest measured chart-decomp-lib - REJECTED, two implementations of one pattern is how they drift, and EM-6 D1 found exactly that when a study private copy of the swing rule was wrong on 906 of 5,672 bars; (C) A BROKEN S/R LEVEL WITH ROLE REVERSAL computed in-process - CHOSEN. OPTION C IS NOT A COMPROMISE, IT IS CH 13 OWN MECHANISM: "pattern resistance - THE MECHANISM EXPLAINS THE PATTERNS" - a neckline works as resistance BECAUSE it is a broken support level, not because it belongs to an H&amp;S. Anchoring on the level is closer to the stated cause and drops the pattern-detector dependency entirely. It also pairs with shipped code: SR_BREAKOUT fires when a level breaks and EM-7 fires when price RETURNS to that same level - one level object, two entries, the second being the register "second chance". SCOPE COST STATED PLAINLY: the TRENDLINE throwback is OUT OF SCOPE and it is the half E&amp;M rate highest ("pullbacks follow trendline breaks MORE frequently than pattern breaks and stop MORE exactly at the old line - no one knows why"). It needs a trendline engine = EM-5 (#65), not built. So EM-7 tests the WEAKER of the book two claims and the result must be reported as such, not as a verdict on the throwback idea. Also noted: the harness compute_sr_levels is a bare swing-cluster with strength:1 carrying NONE of EM-2 break history or role reversal (and EM-2 S9 consumer switch never shipped, so sr_bounce_breakout does not read role_reversed/effective_type either), so that logic must be added in-process. market_features.py exists for exactly this - its docstring says the harness cannot make per-bar HTTP calls so these functions replicate analysis-service concepts from raw bars - so a replica is the ESTABLISHED pattern, but FR-EM-T7 requires asserting agreement with analysis-service sr_volume.detect_breaks, because role ALTERNATION is where EM-2 S5 already got it wrong once. BENCHMARK (C4) is the register one - entry quality vs TAKING THE BREAKOUT ITSELF - as three arms (enter at the break / wait for the throwback / wait for the 40% retracement). PRE-REGISTERED CRITERION: net P&amp;L PER BREAKOUT OPPORTUNITY, counting declined opportunities as ZERO rather than excluding them, symbol-clustered. Reporting average entry price alone is INVALID - a rule that only fills on the best 20% of setups always shows a better average fill while making less money. The FREQUENCY question is a deliverable in its own right (how often does price return to a broken level within N bars, against a matched random-entry null, ordered across boundary types to test E&amp;M relative claim). E&amp;M Return-Line NEGATIVE (a return line does NOT act as support after an upside break) is the useful control: a study that finds throwbacks everywhere has measured something else. HONEST PRIOR: better than EM-6, worse than EM-1. For - the mechanism is the one E&amp;M EXPLAIN rather than assert, and EM-2 established that LEVELS ARE REAL on this data. Against - price returns to a recently broken level OFTEN BY CHANCE (H-T6 null-FPR is for exactly that), and EM-2 closing result is the direct warning: the levels were real and EVERY ELABORATION on them failed. EM-7 is another elaboration on the same levels. NO DB CHANGE. NEXT: Phase 2 plan.  || PHASE 2 PLAN DONE 2026-10-22, docs/implementation_plan_em7_throwback.md. Tasks T0-T5 with TWO gates, front-loaded so TWO working sessions decide whether the remaining three are worth running - the structure that closed EM-6 in three sessions instead of nine. FOUR SRS QUESTIONS SETTLED. (Q3) The two triggers are MUTUALLY EXCLUSIVE MODES (OFF / BAND / RETRACE_40 / EITHER) so they cannot make each other unobservable - the #83 bug class, where capping severities made #82 override structurally unreachable. EITHER is E&amp;M own wording ("whichever comes first") and so is the arm that would ship, but measured alone it cannot say which half does the work, so all three are arms and EITHER is justified only if it beats BOTH singles. (Q1) The proximity band is measured not chosen, in ATR UNITS not percent for the cross-symbol comparability EM-9 established and EM-2 S5/S6 reuse: sweep {0.25, 0.5, 1.0} ATR, primary 0.5. (Q2) Staleness window sweep {20, 60, 120} bars, primary 60. THE TRAP BOTH OF THOSE CARRY, NAMED IN ADVANCE: a wider band and a longer window each find more throwbacks TRIVIALLY, so the T2 null must be matched on BAND AND WINDOW, not merely direction (the EM-2 matched-distance lesson). An unmatched null would measure how generous the band is, not whether throwbacks exist. (Q4) E&amp;M ordering claim (trendline &gt; H&amp;S &gt; double top) is NOT TESTABLE in this scope and NO PROXY IS INVENTED: classifying a level into a pattern family needs a pattern detector, which the SRS rejected, and the trendline arm needs EM-5. Two orderings that ARE available in-process are pre-registered instead - by LEVEL STRENGTH (touch count, since EM-2 established touches are what carry information about a level) and by BREAK DIRECTION (support broken down vs resistance broken up; E&amp;M Return-Line asymmetry suggests they are not mirrors and #85/#86 already found a long/short asymmetry here). GATE 1 IS T2 AND IT NEEDS NO DETECTOR AND NO PIPELINE CHANGE - only T1 and the #87 deep history. It measures BOTH of E&amp;M claims: FREQUENCY (how often price returns to a broken level in the window) and EXACTNESS ("pullbacks stop MORE EXACTLY at the old line", measured as the distribution of OVERSHOOT beyond the level in ATR units - a second independent reading of the same claim, and cheap). Criterion: against a band- AND window-matched random-entry null, the return rate must be HIGHER and the overshoot SMALLER at the primary (0.5 ATR, 60 bar) setting, symbol-clustered. Clustering by SYMBOL is right here and would have been wrong at EM-6 - a level is a per-symbol object. If neither holds, STOP and close #67: a throwback that happens no more often than chance and stops no more precisely is a random limit order with a story attached. T2 also produces the FILL RATE that T4 benchmark needs, which is the second reason it comes first. GATE 2 IS T4: three arms on the SAME breakouts (enter at the break = today SR_BREAKOUT / wait for the throwback / wait for the 40% retracement), criterion = net P&amp;L PER BREAKOUT OPPORTUNITY with declined opportunities counted as ZERO, symbol-clustered, fill rate reported beside it. AVERAGE ENTRY PRICE ALONE IS EXPLICITLY NOT ACCEPTED AS EVIDENCE - a rule that fills only on the best 20% of setups always shows a better average fill while making less money, and it is written into the plan because it is the number that will look most persuasive and mean least. STANDING RISK RECORDED FIRST: this is ANOTHER ELABORATION ON EM-2 LEVELS AND EVERY PREVIOUS ONE FAILED. EM-2 closed on a documented negative - the levels were real (every arm beat a matched-distance null) and NO EM-2 measure beat simply counting touches. T2 null exists because that history says the base rate here is high. Also: if T2 returns a null it is a null on PATTERN-BOUNDARY throwbacks, NOT on E&amp;M trendline claim, and the write-up must not overstate it. NEXT: T0 (roadmap rows, XS) then T1 (break-aware levels in-process, tests first incl. H-T4 role alternation and H-T8 replica agreement with analysis-service).</t>
+          <t>midtrend.py has PCT_RETRACEMENT off the swing and LONG_MA_REACTION but nothing anchored to a broken pattern boundary, so a missed breakout stays missed. failed_signal.py covers the opposite case. Benchmark: entry quality vs taking the breakout itself.  || PHASE 1 DESIGN DONE 2026-10-22, docs/SRS_edwards_magee_throwback.md v1.0 (FR-EM-T1..T8, EC-T1..T6, H-T1..H-T8). NOTHING BUILT. FEASIBILITY WAS DECIDED FIRST, BECAUSE EM-8 M3 JUST SHOWED WHY: MEASURED_MOVE was dead code reading a key no detector ever put in signal evidence, so the mechanism could not be measured at all. EM-7 wants a BROKEN PATTERN BOUNDARY at signal time, which is the same class of dependency. Three options weighed: (A) ai-insights patterns_data, already fetched at orchestrator.py:119 - works live but the harness makes NO per-bar HTTP calls by design, so it is UNMEASURABLE and cannot clear C4 - REJECTED as the MEASURED_MOVE trap exactly; (B) add chart-decomp-lib to decision-helper (it has head_shoulders.py, double.py, triangle.py; chart-decomp-service and event-reaction-service already depend on it) - measurable, but production would run ai-insights detector while the backtest measured chart-decomp-lib - REJECTED, two implementations of one pattern is how they drift, and EM-6 D1 found exactly that when a study private copy of the swing rule was wrong on 906 of 5,672 bars; (C) A BROKEN S/R LEVEL WITH ROLE REVERSAL computed in-process - CHOSEN. OPTION C IS NOT A COMPROMISE, IT IS CH 13 OWN MECHANISM: "pattern resistance - THE MECHANISM EXPLAINS THE PATTERNS" - a neckline works as resistance BECAUSE it is a broken support level, not because it belongs to an H&amp;S. Anchoring on the level is closer to the stated cause and drops the pattern-detector dependency entirely. It also pairs with shipped code: SR_BREAKOUT fires when a level breaks and EM-7 fires when price RETURNS to that same level - one level object, two entries, the second being the register "second chance". SCOPE COST STATED PLAINLY: the TRENDLINE throwback is OUT OF SCOPE and it is the half E&amp;M rate highest ("pullbacks follow trendline breaks MORE frequently than pattern breaks and stop MORE exactly at the old line - no one knows why"). It needs a trendline engine = EM-5 (#65), not built. So EM-7 tests the WEAKER of the book two claims and the result must be reported as such, not as a verdict on the throwback idea. Also noted: the harness compute_sr_levels is a bare swing-cluster with strength:1 carrying NONE of EM-2 break history or role reversal (and EM-2 S9 consumer switch never shipped, so sr_bounce_breakout does not read role_reversed/effective_type either), so that logic must be added in-process. market_features.py exists for exactly this - its docstring says the harness cannot make per-bar HTTP calls so these functions replicate analysis-service concepts from raw bars - so a replica is the ESTABLISHED pattern, but FR-EM-T7 requires asserting agreement with analysis-service sr_volume.detect_breaks, because role ALTERNATION is where EM-2 S5 already got it wrong once. BENCHMARK (C4) is the register one - entry quality vs TAKING THE BREAKOUT ITSELF - as three arms (enter at the break / wait for the throwback / wait for the 40% retracement). PRE-REGISTERED CRITERION: net P&amp;L PER BREAKOUT OPPORTUNITY, counting declined opportunities as ZERO rather than excluding them, symbol-clustered. Reporting average entry price alone is INVALID - a rule that only fills on the best 20% of setups always shows a better average fill while making less money. The FREQUENCY question is a deliverable in its own right (how often does price return to a broken level within N bars, against a matched random-entry null, ordered across boundary types to test E&amp;M relative claim). E&amp;M Return-Line NEGATIVE (a return line does NOT act as support after an upside break) is the useful control: a study that finds throwbacks everywhere has measured something else. HONEST PRIOR: better than EM-6, worse than EM-1. For - the mechanism is the one E&amp;M EXPLAIN rather than assert, and EM-2 established that LEVELS ARE REAL on this data. Against - price returns to a recently broken level OFTEN BY CHANCE (H-T6 null-FPR is for exactly that), and EM-2 closing result is the direct warning: the levels were real and EVERY ELABORATION on them failed. EM-7 is another elaboration on the same levels. NO DB CHANGE. NEXT: Phase 2 plan.  || PHASE 2 PLAN DONE 2026-10-22, docs/implementation_plan_em7_throwback.md. Tasks T0-T5 with TWO gates, front-loaded so TWO working sessions decide whether the remaining three are worth running - the structure that closed EM-6 in three sessions instead of nine. FOUR SRS QUESTIONS SETTLED. (Q3) The two triggers are MUTUALLY EXCLUSIVE MODES (OFF / BAND / RETRACE_40 / EITHER) so they cannot make each other unobservable - the #83 bug class, where capping severities made #82 override structurally unreachable. EITHER is E&amp;M own wording ("whichever comes first") and so is the arm that would ship, but measured alone it cannot say which half does the work, so all three are arms and EITHER is justified only if it beats BOTH singles. (Q1) The proximity band is measured not chosen, in ATR UNITS not percent for the cross-symbol comparability EM-9 established and EM-2 S5/S6 reuse: sweep {0.25, 0.5, 1.0} ATR, primary 0.5. (Q2) Staleness window sweep {20, 60, 120} bars, primary 60. THE TRAP BOTH OF THOSE CARRY, NAMED IN ADVANCE: a wider band and a longer window each find more throwbacks TRIVIALLY, so the T2 null must be matched on BAND AND WINDOW, not merely direction (the EM-2 matched-distance lesson). An unmatched null would measure how generous the band is, not whether throwbacks exist. (Q4) E&amp;M ordering claim (trendline &gt; H&amp;S &gt; double top) is NOT TESTABLE in this scope and NO PROXY IS INVENTED: classifying a level into a pattern family needs a pattern detector, which the SRS rejected, and the trendline arm needs EM-5. Two orderings that ARE available in-process are pre-registered instead - by LEVEL STRENGTH (touch count, since EM-2 established touches are what carry information about a level) and by BREAK DIRECTION (support broken down vs resistance broken up; E&amp;M Return-Line asymmetry suggests they are not mirrors and #85/#86 already found a long/short asymmetry here). GATE 1 IS T2 AND IT NEEDS NO DETECTOR AND NO PIPELINE CHANGE - only T1 and the #87 deep history. It measures BOTH of E&amp;M claims: FREQUENCY (how often price returns to a broken level in the window) and EXACTNESS ("pullbacks stop MORE EXACTLY at the old line", measured as the distribution of OVERSHOOT beyond the level in ATR units - a second independent reading of the same claim, and cheap). Criterion: against a band- AND window-matched random-entry null, the return rate must be HIGHER and the overshoot SMALLER at the primary (0.5 ATR, 60 bar) setting, symbol-clustered. Clustering by SYMBOL is right here and would have been wrong at EM-6 - a level is a per-symbol object. If neither holds, STOP and close #67: a throwback that happens no more often than chance and stops no more precisely is a random limit order with a story attached. T2 also produces the FILL RATE that T4 benchmark needs, which is the second reason it comes first. GATE 2 IS T4: three arms on the SAME breakouts (enter at the break = today SR_BREAKOUT / wait for the throwback / wait for the 40% retracement), criterion = net P&amp;L PER BREAKOUT OPPORTUNITY with declined opportunities counted as ZERO, symbol-clustered, fill rate reported beside it. AVERAGE ENTRY PRICE ALONE IS EXPLICITLY NOT ACCEPTED AS EVIDENCE - a rule that fills only on the best 20% of setups always shows a better average fill while making less money, and it is written into the plan because it is the number that will look most persuasive and mean least. STANDING RISK RECORDED FIRST: this is ANOTHER ELABORATION ON EM-2 LEVELS AND EVERY PREVIOUS ONE FAILED. EM-2 closed on a documented negative - the levels were real (every arm beat a matched-distance null) and NO EM-2 measure beat simply counting touches. T2 null exists because that history says the base rate here is high. Also: if T2 returns a null it is a null on PATTERN-BOUNDARY throwbacks, NOT on E&amp;M trendline claim, and the write-up must not overstate it. NEXT: T0 (roadmap rows, XS) then T1 (break-aware levels in-process, tests first incl. H-T4 role alternation and H-T8 replica agreement with analysis-service).  || T0 DONE 2026-10-22: Feature Inventory row added for EM-7 (In Progress), FR-EM-T1..T8 / EC-T1..T6 / H-T1..H-T8 recorded, where-it-lives named (market_features.py for T1, signal/trend/ for T3). No code. NEXT: T1.</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -11528,7 +11565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F212"/>
+  <dimension ref="A1:F213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17544,6 +17581,38 @@
         </is>
       </c>
       <c r="F212" s="4" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="120" customHeight="1">
+      <c r="A213" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t>EM-7 T0 - roadmap rows and requirement wiring (XS, no code)</t>
+        </is>
+      </c>
+      <c r="C213" s="4" t="inlineStr">
+        <is>
+          <t>ROADMAP: NEW Feature Inventory row for EM-7 (In Progress) carrying the anchor decision and the scope cost; #67 Backlog row updated with T0 done. No code touched.</t>
+        </is>
+      </c>
+      <c r="D213" s="4" t="inlineStr">
+        <is>
+          <t>Nothing measured or learned - this is the bookkeeping task the plan budgeted as XS, kept separate so T1 starts from a clean, recorded baseline. The Feature Inventory row deliberately carries the two things a future reader needs and would not find in the code: WHY the anchor is a broken S/R level rather than a pattern neckline (options A and B are unmeasurable or run a different detector than production), and WHAT that cost (the trendline half, which E&amp;M rate highest, needs EM-5). Added an idempotence guard so re-running T0 raises instead of duplicating the row.</t>
+        </is>
+      </c>
+      <c r="E213" s="4" t="inlineStr">
+        <is>
+          <t>T0 DONE. NEXT IS T1: break-aware levels in backtest/market_features.py - each level carrying the bar it was decisively penetrated, the direction, and its effective type after the break. Tests FIRST: H-T4 role ALTERNATION (the EM-2 S5 bug: an oscillating series must not report a support as broken upward on every rally - found there only by building a genuinely quiet fixture rather than trusting an oscillating one), H-T1 causality (appending future bars moves no past break), H-T8 agreement with analysis-service sr_volume.detect_breaks on shared fixtures, H-T7 bound-default mutation check (eighth instance). Then GATE 1 at T2. 20 backlog items open; #67 In Progress.</t>
+        </is>
+      </c>
+      <c r="F213" s="4" t="inlineStr">
         <is>
           <t>None.</t>
         </is>

</xml_diff>

<commit_message>
docs(roadmap): session log 2026-10-25 — auth fixes moved onto stockpredict
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Inventory" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech Debt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions Log" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Feature Inventory" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Roadmap" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Tech Debt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sessions Log" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Architecture" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Feature Inventory'!$A$1:$G$110</definedName>
@@ -11762,7 +11762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F230"/>
+  <dimension ref="A1:F231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18357,6 +18357,38 @@
       <c r="F230" s="4" t="inlineStr">
         <is>
           <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B231" s="4" t="inlineStr">
+        <is>
+          <t>Fresh clone landed on stale main; moved auth fixes onto stockpredict</t>
+        </is>
+      </c>
+      <c r="C231" s="4" t="inlineStr">
+        <is>
+          <t>Fresh clone checked out main (108 commits behind stockpredict). On stockpredict: 8a80fe40 login error text 'Invalid username/email or password' + formatApiError() for FastAPI 422 list detail + api.test.js + MIGRATION.md new tunnel ID 90a553cf; 8a2cc638 UserLogin field email -&gt; username with AliasChoices('username','email') (old clients keep working), frontend sends username. A stock-data upsert/dup-column fix made on main was dropped - stockpredict already had both.</t>
+        </is>
+      </c>
+      <c r="D231" s="4" t="inlineStr">
+        <is>
+          <t>Always clone/switch to the stockpredict branch - main is stale. Images built + stack started this session came from main code; need a rebuild from stockpredict. Local main still holds 5 unpushed commits that should NOT be pushed (superseded).</t>
+        </is>
+      </c>
+      <c r="E231" s="4" t="inlineStr">
+        <is>
+          <t>DONE: auth tests 106 passed (with branch stock-common), frontend api/httpClient 7 passed. NOT pushed - no GitHub credentials on this box (install gh + gh auth login). Next: push stockpredict; rebuild + redeploy from stockpredict; reset local main to origin/main; then backlog #59/#48/#91, decisions #98/#49.</t>
+        </is>
+      </c>
+      <c r="F231" s="4" t="inlineStr">
+        <is>
+          <t>No GitHub auth on this machine. /etc/cloudflared backup + cloudflared start need sudo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(stock-data): #59 — dividends read from VCI corporate events
No vnstock 4.0.7 source exposes Company.dividends(), so /companies/{symbol}/dividends
returned [] for every symbol. VCI's corporate-events feed carries them:

- fall back to data_source._fetch_events(event_codes='DIV,ISS'), paged from 2000.
  The public events() returns one page of 50 across all event types, so director
  dealings crowded dividends out (FPT: 4 cash dividends vs 40 available).
- keep DIV (cash) and ISS titled 'Stock dividend' / 'Bonus Issue'; drop ESOP,
  rights issues, private placements, bond conversions. VCI tags all of them
  category=DIVIDEND, so the English title is the only discriminator.
- map to the keys CompanyDividents.js already reads (title, exrightDate,
  issueDate=payout, ratio, value, eventType/eventTypeEn), newest first.

Live: FPT 58 rows back to 2007, VNM 58 back to 2006. 264 passed (+4), ruff clean.
Unblocks #58.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -9794,12 +9794,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Found while investigating #56. vnstock 4.0.7 supports KBS/VCI/MSN/FMP — TCBS is gone, and VCI's Company exposes no dividends(). The endpoint is dead against the configured source. Also blocks #58, which needs an ex-date list.</t>
+          <t>Found while investigating #56. vnstock 4.0.7 supports KBS/VCI/MSN/FMP — TCBS is gone, and VCI's Company exposes no dividends(). The endpoint is dead against the configured source. Also blocks #58, which needs an ex-date list. || DONE 2026-10-25: no 4.0.7 source has Company.dividends(), but VCI corporate events carry them. get_company_dividends_data now falls back to data_source._fetch_events(event_codes='DIV,ISS', from_date=2000, paged 200) - public events() returns ONE page of 50 across all event types, so director deals crowded dividends out (FPT: 4 cash divs vs 19+ via DIV,ISS). Kept: DIV (cash) + ISS titled 'Stock dividend' / 'Bonus Issue'; dropped ESOP, rights, private placement, convertible, merger (VCI tags ALL of them category=DIVIDEND, so title is the only discriminator). Mapped to the frontend's existing keys (title, exrightDate, issueDate=payout, ratio, value, eventType/En) + recordDate, titleEn, eventCode. Live: FPT 58 rows back to 2007, VNM 58 back to 2006 (were 0). stock-data 264 passed (+4), ruff clean. UNBLOCKS #58 (ex-date list now available).</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -11762,7 +11762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F231"/>
+  <dimension ref="A1:F232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18389,6 +18389,38 @@
       <c r="F231" s="4" t="inlineStr">
         <is>
           <t>No GitHub auth on this machine. /etc/cloudflared backup + cloudflared start need sudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B232" s="4" t="inlineStr">
+        <is>
+          <t>#59 fixed - dividends endpoint was empty for every symbol</t>
+        </is>
+      </c>
+      <c r="C232" s="4" t="inlineStr">
+        <is>
+          <t>stock_service.get_company_dividends_data: when the source lacks dividends() (VCI), read DIV/ISS corporate events via _fetch_events, paged; new _dividend_events_to_records maps them to the frontend's keys. 4 tests (mapper, missing fields, fallback call, paging). Rebuilt + redeployed stock-data-service only.</t>
+        </is>
+      </c>
+      <c r="D232" s="4" t="inlineStr">
+        <is>
+          <t>VCI events(): public method is hardwired to 1 page x 50 rows across ALL event types; the private _fetch_events takes event_codes/from_date/page/size. Relying on a private method is acceptable only because vnstock is frozen at vendored 4.0.7 (#96/#98) - revisit if that changes. VCI tags every DIV/ISS row category=DIVIDEND incl. ESOP, so classification is by eventTitleEn.</t>
+        </is>
+      </c>
+      <c r="E232" s="4" t="inlineStr">
+        <is>
+          <t>DONE + verified live: FPT 58 dividend rows (2007-&gt;), VNM 58 (2006-&gt;); stock-data 264 passed, ruff clean. Committed, NOT pushed. Next candidates: #48 (Price Board stale intraday), #91 (dead market_indices table), #58 (cash-dividend adjustment - now unblocked by #59). Owner decisions still open: #98, #49.</t>
+        </is>
+      </c>
+      <c r="F232" s="4" t="inlineStr">
+        <is>
+          <t>None.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(stock-data): #48 — refresh a stale price board, not only an empty one
The board was refreshed only when its DB group was empty, and the nightly
refresh runs at 01:00 with the market closed, so matchPrice/change sat at
0/null all trading day unless an admin hit /priceboards/refresh.

- price_board_is_stale(): in session (Mon-Fri 09:00-15:00 ICT) stale when
  older than PRICE_BOARD_MAX_AGE_SECONDS (default 60 — one Vietcap POST, no
  vnstock quota); outside session stale when taken before the last close.
- get_price_board refreshes stale groups under a per-group lock, so
  concurrent readers cause one refresh.
- a failed refresh serves the existing rows instead of blanking the board.

Verified live: backdated VN30 refreshed on the next read, the following read
was a cache hit; 30/30 rows priced. 275 passed (+11), ruff clean.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stockpredict/ROADMAP.xlsx
+++ b/stockpredict/ROADMAP.xlsx
@@ -9409,12 +9409,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Price Board shows 0 / N/A for match price and change during trading hours.</t>
+          <t>Price Board shows 0 / N/A for match price and change during trading hours. || DONE 2026-10-25: get_price_board now refreshes when the cached group is STALE, not only when empty. price_board_is_stale(): in session (Mon-Fri 09:00-15:00 ICT, fixed UTC+7) stale if older than PRICE_BOARD_MAX_AGE_SECONDS (default 60; one Vietcap POST, no vnstock quota); outside session stale if taken before the most recent close (so after-hours/weekends show the last session's final prices, and the 01:00 snapshot after a close is still fresh). Per-group asyncio lock so concurrent readers trigger one refresh. A failed refresh serves the stale rows instead of blanking the board. Holidays not modelled (at most one refetch per max-age). Verified live: VN30 backdated to Fri 01:00 -&gt; 1st request refreshed (0.88s, 'stale ... refreshing' logged), 2nd served from cache (0.01s); 30/30 rows with matchPrice. 275 passed (+11), ruff clean.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -11762,7 +11762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F232"/>
+  <dimension ref="A1:F233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18419,6 +18419,38 @@
         </is>
       </c>
       <c r="F232" s="4" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B233" s="4" t="inlineStr">
+        <is>
+          <t>#48 fixed - Price Board was showing 0/N/A all trading day</t>
+        </is>
+      </c>
+      <c r="C233" s="4" t="inlineStr">
+        <is>
+          <t>stock_service.get_price_board: staleness-aware refresh (new price_board_is_stale + per-group lock + keep stale rows on failed refresh); config PRICE_BOARD_MAX_AGE_SECONDS=60. 11 tests (9 staleness cases incl. the 01:00 bug, weekend, overnight; refresh-when-stale; stale-survives-failed-refresh). Existing cache-hit test now pins the clock. Rebuilt + redeployed stock-data-service only.</t>
+        </is>
+      </c>
+      <c r="D233" s="4" t="inlineStr">
+        <is>
+          <t>Staleness is per session, not just age: outside trading hours the right question is 'was this taken after the last close?', which also makes the 01:00 nightly snapshot correct overnight. Frontend does not poll the board, so per-request staleness is enough; single uvicorn worker, so an in-process lock prevents duplicate refreshes.</t>
+        </is>
+      </c>
+      <c r="E233" s="4" t="inlineStr">
+        <is>
+          <t>DONE + verified live (Sunday, so the outside-session path; in-session path covered by unit tests only - re-check on a weekday 09:00-15:00 ICT). Committed, NOT pushed. Next candidates: #91 (dead market_indices table), #58 (cash-dividend adjustment, unblocked by #59). Owner decisions: #98, #49.</t>
+        </is>
+      </c>
+      <c r="F233" s="4" t="inlineStr">
         <is>
           <t>None.</t>
         </is>

</xml_diff>